<commit_message>
docs: accept M1-T6 - review record (PASS), domain-model + testing-strategy updates, follow-ups triaged, dispatch M1-T7
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andy\OneDrive\006_Smart Kitchen App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{808FDF22-DB6E-4D5D-B36F-3007FBB05609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6A6150D2-EB8F-48C7-8C0D-C5B64D982EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{28AEF9BF-1F49-4F7C-87F4-15C43A581099}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7369F377-974A-4F18-B7AC-C241A8F4F966}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="169">
   <si>
     <t>ID</t>
   </si>
@@ -275,28 +275,28 @@
     <t>M1-T4 (done)</t>
   </si>
   <si>
+    <t>Done - accepted &amp; squash-merged 2026-09-14</t>
+  </si>
+  <si>
+    <t>Review: PASS no fixes (488 probes + 4500 fuzz runs; 0 leaks); +136 tests; pre-M4 gate (a) closed; D-018 batch item 1 of 5</t>
+  </si>
+  <si>
+    <t>M1-T7</t>
+  </si>
+  <si>
+    <t>Correction-rate telemetry: SQL view + read function (north-star KPI)</t>
+  </si>
+  <si>
+    <t>Read-only view + repository read; metric definition fixed in ticket</t>
+  </si>
+  <si>
+    <t>Tenancy (security_invoker view; ADR-003 rule 3) + exact KPI counting</t>
+  </si>
+  <si>
+    <t>M1-T2 (done)</t>
+  </si>
+  <si>
     <t>In progress - dispatched 2026-09-14</t>
-  </si>
-  <si>
-    <t>D-018 batch item 1 of 5</t>
-  </si>
-  <si>
-    <t>M1-T7</t>
-  </si>
-  <si>
-    <t>Correction-rate telemetry: SQL view + read function (north-star KPI)</t>
-  </si>
-  <si>
-    <t>Read-only view + repository read; metric definition fixed in ticket</t>
-  </si>
-  <si>
-    <t>Tenancy (security_invoker view; ADR-003 rule 3) + exact KPI counting</t>
-  </si>
-  <si>
-    <t>M1-T2 (done)</t>
-  </si>
-  <si>
-    <t>Queued (after M1-T6)</t>
   </si>
   <si>
     <t>D-018 batch item 2 of 5</t>
@@ -939,7 +939,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0827BC3-D30C-4B89-B36C-D8D3C0B8B03F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CC121D0-1224-4834-87A0-810685210070}">
   <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1361,7 +1361,9 @@
       <c r="K10" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="L10" s="2"/>
+      <c r="L10" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="M10" s="2" t="s">
         <v>85</v>
       </c>
@@ -1833,7 +1835,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M22" xr:uid="{D0827BC3-D30C-4B89-B36C-D8D3C0B8B03F}"/>
+  <autoFilter ref="A1:M22" xr:uid="{3CC121D0-1224-4834-87A0-810685210070}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M1-T7 - review record (PASS), correction-rate KPI definition in ARCHITECTURE s8, follow-ups triaged, dispatch M1-T8
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andy\OneDrive\006_Smart Kitchen App\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6A6150D2-EB8F-48C7-8C0D-C5B64D982EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E30FE0FC-E91C-4039-A2E6-0453ABE0B349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7369F377-974A-4F18-B7AC-C241A8F4F966}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CFA4A46E-8A6D-4E87-A5D6-522742257B43}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="168">
   <si>
     <t>ID</t>
   </si>
@@ -296,28 +296,25 @@
     <t>M1-T2 (done)</t>
   </si>
   <si>
+    <t>Review: PASS no fixes (16 tenancy probes on real Postgres; 9 mutations); 625 tests w/ DB; KPI definition in ARCHITECTURE s8; D-018 batch item 2 of 5</t>
+  </si>
+  <si>
+    <t>M1-T8</t>
+  </si>
+  <si>
+    <t>Lot-selection policy for consumption (FEFO/FIFO planner)</t>
+  </si>
+  <si>
+    <t>Inventory arithmetic splitting a decrease across lots (rule-23 list)</t>
+  </si>
+  <si>
+    <t>Probe ordering ties; undated/expired lots; exhaustion; reserved-key namespace</t>
+  </si>
+  <si>
+    <t>M1-T1 (done)</t>
+  </si>
+  <si>
     <t>In progress - dispatched 2026-09-14</t>
-  </si>
-  <si>
-    <t>D-018 batch item 2 of 5</t>
-  </si>
-  <si>
-    <t>M1-T8</t>
-  </si>
-  <si>
-    <t>Lot-selection policy for consumption (FEFO/FIFO planner)</t>
-  </si>
-  <si>
-    <t>Inventory arithmetic splitting a decrease across lots (rule-23 list)</t>
-  </si>
-  <si>
-    <t>Probe ordering ties; undated/expired lots; exhaustion; reserved-key namespace</t>
-  </si>
-  <si>
-    <t>M1-T1 (done)</t>
-  </si>
-  <si>
-    <t>Queued (after M1-T7)</t>
   </si>
   <si>
     <t>D-018 batch item 3 of 5; FEFO default PROPOSED</t>
@@ -939,7 +936,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CC121D0-1224-4834-87A0-810685210070}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4309569D-CFCE-45CE-9EEF-7E55DF6E6ECE}">
   <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1359,18 +1356,18 @@
         <v>83</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>55</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>33</v>
@@ -1379,7 +1376,7 @@
         <v>72</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>17</v>
@@ -1388,28 +1385,30 @@
         <v>36</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I11" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="K11" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="L11" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M11" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>33</v>
@@ -1418,7 +1417,7 @@
         <v>72</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>17</v>
@@ -1427,28 +1426,28 @@
         <v>18</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>83</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L12" s="2"/>
       <c r="M12" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>33</v>
@@ -1457,7 +1456,7 @@
         <v>72</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>17</v>
@@ -1466,376 +1465,376 @@
         <v>18</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>18</v>
       </c>
       <c r="I13" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="K13" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="L13" s="2"/>
       <c r="M13" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="H14" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="I14" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="I14" s="2" t="s">
+      <c r="J14" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="K14" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F15" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="I15" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="K15" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="L15" s="2"/>
       <c r="M15" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G16" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="I16" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="H16" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>129</v>
-      </c>
       <c r="J16" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G17" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="I17" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="H17" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="I17" s="2" t="s">
+      <c r="J17" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="J17" s="2" t="s">
-        <v>136</v>
-      </c>
       <c r="K17" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>140</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G18" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="I18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="J18" s="2" t="s">
-        <v>143</v>
-      </c>
       <c r="K18" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>146</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>147</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G19" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="I19" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="H19" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="J19" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="K19" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>154</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G20" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>156</v>
-      </c>
       <c r="J20" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>159</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>160</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G21" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="H21" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>162</v>
-      </c>
       <c r="J21" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>164</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>165</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G22" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="I22" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="H22" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="J22" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M22" xr:uid="{3CC121D0-1224-4834-87A0-810685210070}"/>
+  <autoFilter ref="A1:M22" xr:uid="{4309569D-CFCE-45CE-9EEF-7E55DF6E6ECE}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M1-T8 - review record (PASS after fixes), OQ-1 FEFO PROPOSED default, single-read rule in testing-strategy, follow-ups triaged, dispatch M1-T9
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andy\OneDrive\006_Smart Kitchen App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E30FE0FC-E91C-4039-A2E6-0453ABE0B349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9776CD0E-D949-4F8B-AFDB-D20285533021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CFA4A46E-8A6D-4E87-A5D6-522742257B43}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{48AC658A-E624-4F30-A356-C203B82B3F74}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="168">
   <si>
     <t>ID</t>
   </si>
@@ -314,10 +314,10 @@
     <t>M1-T1 (done)</t>
   </si>
   <si>
-    <t>In progress - dispatched 2026-09-14</t>
-  </si>
-  <si>
-    <t>D-018 batch item 3 of 5; FEFO default PROPOSED</t>
+    <t>Done - accepted &amp; squash-merged 2026-09-15</t>
+  </si>
+  <si>
+    <t>Review: PASS WITH FIXES (3 hand-built-input hardenings) -&gt; re-review PASS; 17 mutations 15 killed; +35 tests; FEFO default PROPOSED (OQ-1); D-018 batch item 3 of 5</t>
   </si>
   <si>
     <t>M1-T9</t>
@@ -332,7 +332,7 @@
     <t>Concurrency-sensitive inventory updates; business conflicts must never be retried</t>
   </si>
   <si>
-    <t>Queued (after M1-T8)</t>
+    <t>In progress - dispatched 2026-09-15</t>
   </si>
   <si>
     <t>D-018 batch item 4 of 5</t>
@@ -936,7 +936,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4309569D-CFCE-45CE-9EEF-7E55DF6E6ECE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD456B64-B1DC-4D95-91DD-0C73E3B0CF6F}">
   <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1440,7 +1440,9 @@
       <c r="K12" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="L12" s="2"/>
+      <c r="L12" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="M12" s="2" t="s">
         <v>97</v>
       </c>
@@ -1834,7 +1836,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M22" xr:uid="{4309569D-CFCE-45CE-9EEF-7E55DF6E6ECE}"/>
+  <autoFilter ref="A1:M22" xr:uid="{AD456B64-B1DC-4D95-91DD-0C73E3B0CF6F}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M1-T9 - review record (PASS after fix), ticket M1-T11 (pre-existing aborted-COMMIT data-loss defect, not dispatched), M1-T10 item (m)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andy\OneDrive\006_Smart Kitchen App\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9776CD0E-D949-4F8B-AFDB-D20285533021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{05039A3E-831B-4EAE-92ED-F485611D0B40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{48AC658A-E624-4F30-A356-C203B82B3F74}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{3DCD62A0-B491-49C6-95D9-223417B7811A}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -936,7 +936,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD456B64-B1DC-4D95-91DD-0C73E3B0CF6F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EE26DEF-631C-4215-A0C2-377FA596193B}">
   <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1836,7 +1836,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M22" xr:uid="{AD456B64-B1DC-4D95-91DD-0C73E3B0CF6F}"/>
+  <autoFilter ref="A1:M22" xr:uid="{9EE26DEF-631C-4215-A0C2-377FA596193B}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: M1-T9 acceptance follow-through - M1-T11 ticket text, STATUS rows, tracker row (omitted from 8421b47 by a failed scripted edit)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{05039A3E-831B-4EAE-92ED-F485611D0B40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{35196592-FF24-46A5-8C3E-28AE818D58E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{3DCD62A0-B491-49C6-95D9-223417B7811A}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{B4F1D945-0C5F-4C08-BA47-150263E9DF3D}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$23</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="174">
   <si>
     <t>ID</t>
   </si>
@@ -332,10 +332,28 @@
     <t>Concurrency-sensitive inventory updates; business conflicts must never be retried</t>
   </si>
   <si>
-    <t>In progress - dispatched 2026-09-15</t>
-  </si>
-  <si>
-    <t>D-018 batch item 4 of 5</t>
+    <t>Review: PASS WITH FIXES (pin assumeRole across retries) -&gt; re-review PASS on real Postgres; no double-apply; 697 tests w/ DB; D-018 batch item 4 of 5</t>
+  </si>
+  <si>
+    <t>M1-T11</t>
+  </si>
+  <si>
+    <t>Ledger write path: aborted-transaction COMMIT silently discards work (pre-existing defect)</t>
+  </si>
+  <si>
+    <t>Ledger write-path transaction semantics (rule-23 list)</t>
+  </si>
+  <si>
+    <t>Prove no rolled-back-but-reported-success outcome remains</t>
+  </si>
+  <si>
+    <t>M1-T9 (done); before M2 first write handler</t>
+  </si>
+  <si>
+    <t>Not started - awaits PO go (outside D-018 five)</t>
+  </si>
+  <si>
+    <t>Found by M1-T9 review F4; silent data loss in write path; not reachable in prod today</t>
   </si>
   <si>
     <t>M1-T10</t>
@@ -936,8 +954,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EE26DEF-631C-4215-A0C2-377FA596193B}">
-  <dimension ref="A1:M22"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64826885-6B30-4305-853E-E4B903170555}">
+  <dimension ref="A1:M23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -1438,18 +1456,18 @@
         <v>83</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>55</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>33</v>
@@ -1458,160 +1476,160 @@
         <v>72</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="G13" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I13" s="2" t="s">
+      <c r="J13" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="K13" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="L13" s="2"/>
       <c r="M13" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="E14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="H14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I14" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="J14" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F14" s="2" t="s">
+      <c r="K14" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>113</v>
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F15" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="K15" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="L15" s="2"/>
       <c r="M15" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="G16" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="I16" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="H16" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="I16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="J16" s="2" t="s">
-        <v>105</v>
-      </c>
       <c r="K16" s="2" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>132</v>
@@ -1620,139 +1638,139 @@
         <v>2</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>133</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>134</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>135</v>
+        <v>111</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>139</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G18" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="I18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="J18" s="2" t="s">
-        <v>142</v>
-      </c>
       <c r="K18" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G19" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I19" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="H19" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="J19" s="2" t="s">
-        <v>149</v>
-      </c>
       <c r="K19" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>152</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>153</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G20" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="I20" s="2" t="s">
+      <c r="J20" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="J20" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="K20" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2" t="s">
@@ -1767,7 +1785,7 @@
         <v>158</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>159</v>
@@ -1776,67 +1794,106 @@
         <v>2</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>160</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>161</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
+      <c r="M21" s="2" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>157</v>
       </c>
       <c r="K22" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2" t="s">
-        <v>167</v>
+      <c r="D23" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="L23" s="2"/>
+      <c r="M23" s="2" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M22" xr:uid="{9EE26DEF-631C-4215-A0C2-377FA596193B}"/>
+  <autoFilter ref="A1:M23" xr:uid="{64826885-6B30-4305-853E-E4B903170555}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M1-T10 - D-018 batch complete, engineering stopped for PO review; M3-E0-T1..T3 ticketed (not dispatched); review record
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{35196592-FF24-46A5-8C3E-28AE818D58E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{529C48FD-6D8A-4C40-AED0-2DE2BF5626F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{B4F1D945-0C5F-4C08-BA47-150263E9DF3D}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{BE15B04D-E95E-4503-B616-95C501260B92}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$26</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="193">
   <si>
     <t>ID</t>
   </si>
@@ -371,10 +371,67 @@
     <t>M1-T6; M1-T9 (runs last)</t>
   </si>
   <si>
-    <t>Queued (after M1-T9)</t>
-  </si>
-  <si>
-    <t>D-018 batch item 5 of 5; STOP for PO review after acceptance</t>
+    <t>Review: PASS no fixes; all 13 items (a-m) landed; +71 tests (769 w/ DB); D-018 batch COMPLETE - engineering stopped for PO review</t>
+  </si>
+  <si>
+    <t>M3-E0-T1</t>
+  </si>
+  <si>
+    <t>M3 Basic client (UI)</t>
+  </si>
+  <si>
+    <t>M3-E0 UX design gate</t>
+  </si>
+  <si>
+    <t>Prototype completion: missing MVP screens + non-happy states (docs only)</t>
+  </si>
+  <si>
+    <t>HTML/CSS prototype work inside the token system; no product logic</t>
+  </si>
+  <si>
+    <t>Safety copy audit (nine rules; P11; three verdict states)</t>
+  </si>
+  <si>
+    <t>D-019 (done)</t>
+  </si>
+  <si>
+    <t>Not started - awaits PO go</t>
+  </si>
+  <si>
+    <t>Written 2026-09-15; S1/S2/S5/S9/S12 + recipe detail + states + legend/undo/who-did-what</t>
+  </si>
+  <si>
+    <t>M3-E0-T2</t>
+  </si>
+  <si>
+    <t>Safety and provenance copy deck (docs only)</t>
+  </si>
+  <si>
+    <t>Writing to a fixed rule set</t>
+  </si>
+  <si>
+    <t>Reviewed like code vs nine rules / D-017 / P11; coverage vs type unions</t>
+  </si>
+  <si>
+    <t>none (parallel with T1)</t>
+  </si>
+  <si>
+    <t>Becomes the client string table for allergen surfaces</t>
+  </si>
+  <si>
+    <t>M3-E0-T3</t>
+  </si>
+  <si>
+    <t>Token sheet: contrast measurements + scarcity audit (docs only)</t>
+  </si>
+  <si>
+    <t>Measurement and tabulation</t>
+  </si>
+  <si>
+    <t>Check arithmetic; no token drift from prototype</t>
+  </si>
+  <si>
+    <t>Output docs/design/tokens.md ready for the typed token module in M3</t>
   </si>
   <si>
     <t>M2</t>
@@ -954,11 +1011,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64826885-6B30-4305-853E-E4B903170555}">
-  <dimension ref="A1:M23"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F727B3A1-0FCD-42EF-9AD7-D4F9CFBA2ABA}">
+  <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="60.7109375" customWidth="1"/>
@@ -1536,202 +1593,204 @@
         <v>108</v>
       </c>
       <c r="K14" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="M14" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F15" s="2" t="s">
+      <c r="H15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="H15" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="I15" s="2" t="s">
+      <c r="K15" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="L15" s="2"/>
       <c r="M15" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="H16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I16" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>128</v>
-      </c>
       <c r="K16" s="2" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>115</v>
+        <v>18</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>115</v>
+        <v>18</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>115</v>
+        <v>143</v>
       </c>
       <c r="G19" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I19" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H19" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2" t="s">
@@ -1743,157 +1802,274 @@
         <v>150</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="G20" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>154</v>
-      </c>
       <c r="J20" s="2" t="s">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>159</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="G21" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="J21" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="H21" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="K21" s="2" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>164</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>165</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="G22" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I22" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="H22" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="I22" s="2" t="s">
+      <c r="J22" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="J22" s="2" t="s">
-        <v>157</v>
-      </c>
       <c r="K22" s="2" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
+      <c r="M22" s="2" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="L25" s="2"/>
+      <c r="M25" s="2"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="L26" s="2"/>
+      <c r="M26" s="2" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M23" xr:uid="{64826885-6B30-4305-853E-E4B903170555}"/>
+  <autoFilter ref="A1:M26" xr:uid="{F727B3A1-0FCD-42EF-9AD7-D4F9CFBA2ABA}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: D-018a - PO approves M1-T11 then M3-E0-T1/T2 parallel then T3; dispatch M1-T11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{529C48FD-6D8A-4C40-AED0-2DE2BF5626F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2FC1B1BB-24EA-4B19-811C-B6968118E6E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{BE15B04D-E95E-4503-B616-95C501260B92}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{ED68C74F-F6C5-4A6D-A257-B5AB1C895EBF}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="194">
   <si>
     <t>ID</t>
   </si>
@@ -350,7 +350,7 @@
     <t>M1-T9 (done); before M2 first write handler</t>
   </si>
   <si>
-    <t>Not started - awaits PO go (outside D-018 five)</t>
+    <t>In progress - dispatched 2026-09-15 (D-018a)</t>
   </si>
   <si>
     <t>Found by M1-T9 review F4; silent data loss in write path; not reachable in prod today</t>
@@ -395,7 +395,7 @@
     <t>D-019 (done)</t>
   </si>
   <si>
-    <t>Not started - awaits PO go</t>
+    <t>Queued (after M1-T11; T1 and T2 parallel) - D-018a</t>
   </si>
   <si>
     <t>Written 2026-09-15; S1/S2/S5/S9/S12 + recipe detail + states + legend/undo/who-did-what</t>
@@ -429,6 +429,9 @@
   </si>
   <si>
     <t>Check arithmetic; no token drift from prototype</t>
+  </si>
+  <si>
+    <t>Queued (after M3-E0-T1) - D-018a</t>
   </si>
   <si>
     <t>Output docs/design/tokens.md ready for the typed token module in M3</t>
@@ -1011,7 +1014,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F727B3A1-0FCD-42EF-9AD7-D4F9CFBA2ABA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D0CEBCF-B6AD-4250-902E-68357B9C78DF}">
   <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1556,7 +1559,9 @@
       <c r="K13" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="L13" s="2"/>
+      <c r="L13" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="M13" s="2" t="s">
         <v>103</v>
       </c>
@@ -1712,364 +1717,364 @@
         <v>110</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G18" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="H18" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="I18" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="L26" s="2"/>
       <c r="M26" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M26" xr:uid="{F727B3A1-0FCD-42EF-9AD7-D4F9CFBA2ABA}"/>
+  <autoFilter ref="A1:M26" xr:uid="{7D0CEBCF-B6AD-4250-902E-68357B9C78DF}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M1-T11 - review record (PASS after fix), data-model s6 savepoint + COMMIT-tag rules, follow-ups; dispatch M3-E0-T1 and T2 in parallel
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2FC1B1BB-24EA-4B19-811C-B6968118E6E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A563740-2C5A-490B-8213-0426D88A4F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{ED68C74F-F6C5-4A6D-A257-B5AB1C895EBF}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{399FB43B-65D5-4E8F-8F7A-3D6AFDCFBFFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="194">
   <si>
     <t>ID</t>
   </si>
@@ -350,10 +350,10 @@
     <t>M1-T9 (done); before M2 first write handler</t>
   </si>
   <si>
-    <t>In progress - dispatched 2026-09-15 (D-018a)</t>
-  </si>
-  <si>
-    <t>Found by M1-T9 review F4; silent data loss in write path; not reachable in prod today</t>
+    <t>Done - accepted &amp; squash-merged 2026-09-16</t>
+  </si>
+  <si>
+    <t>Review: PASS WITH FIXES (pin fn-thrown-error rollback path; tenancy-leak mutant) -&gt; re-review PASS; F4 repro 0 -&gt; 1 durable row; 786 tests w/ DB</t>
   </si>
   <si>
     <t>M1-T10</t>
@@ -395,7 +395,7 @@
     <t>D-019 (done)</t>
   </si>
   <si>
-    <t>Queued (after M1-T11; T1 and T2 parallel) - D-018a</t>
+    <t>In progress - dispatched 2026-09-16 (parallel)</t>
   </si>
   <si>
     <t>Written 2026-09-15; S1/S2/S5/S9/S12 + recipe detail + states + legend/undo/who-did-what</t>
@@ -1014,7 +1014,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D0CEBCF-B6AD-4250-902E-68357B9C78DF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3548503D-9CFD-4660-ACAF-F97C3AE7563B}">
   <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1641,7 +1641,9 @@
       <c r="K15" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="L15" s="2"/>
+      <c r="L15" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="M15" s="2" t="s">
         <v>118</v>
       </c>
@@ -1680,7 +1682,9 @@
       <c r="K16" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="L16" s="2"/>
+      <c r="L16" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="M16" s="2" t="s">
         <v>124</v>
       </c>
@@ -2074,7 +2078,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M26" xr:uid="{7D0CEBCF-B6AD-4250-902E-68357B9C78DF}"/>
+  <autoFilter ref="A1:M26" xr:uid="{3548503D-9CFD-4660-ACAF-F97C3AE7563B}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M3-E0-T2 - review record (PASS after fixes), R1-R3 nits, canonical caveat aligned in design-direction, follow-ups triaged
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A563740-2C5A-490B-8213-0426D88A4F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA66624F-7371-466C-B2DF-7233A726736C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{399FB43B-65D5-4E8F-8F7A-3D6AFDCFBFFA}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{CA0F7F05-6B46-4102-8D35-67320C61107E}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -416,7 +416,7 @@
     <t>none (parallel with T1)</t>
   </si>
   <si>
-    <t>Becomes the client string table for allergen surfaces</t>
+    <t>Review: PASS WITH FIXES (5 safety-wording defects + 9 smaller) -&gt; re-review PASS; 63/63 codes; binding for M3 string table. Becomes the client string table for allergen surfaces</t>
   </si>
   <si>
     <t>M3-E0-T3</t>
@@ -1014,7 +1014,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3548503D-9CFD-4660-ACAF-F97C3AE7563B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67E6F0A1-0DCD-40C3-A117-E39AF7BCACDB}">
   <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1680,7 +1680,7 @@
         <v>123</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>55</v>
@@ -2078,7 +2078,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M26" xr:uid="{3548503D-9CFD-4660-ACAF-F97C3AE7563B}"/>
+  <autoFilter ref="A1:M26" xr:uid="{67E6F0A1-0DCD-40C3-A117-E39AF7BCACDB}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M3-E0-T1 - review record (PASS after fixes), caveat on the normal-mode blocked row, follow-ups triaged; dispatch M3-E0-T3
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA66624F-7371-466C-B2DF-7233A726736C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3583944-EC0D-4A5A-88B7-86C37381DCD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{CA0F7F05-6B46-4102-8D35-67320C61107E}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{31410C2C-C827-48E9-B149-314833D2161E}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="193">
   <si>
     <t>ID</t>
   </si>
@@ -395,10 +395,7 @@
     <t>D-019 (done)</t>
   </si>
   <si>
-    <t>In progress - dispatched 2026-09-16 (parallel)</t>
-  </si>
-  <si>
-    <t>Written 2026-09-15; S1/S2/S5/S9/S12 + recipe detail + states + legend/undo/who-did-what</t>
+    <t>Review: PASS WITH FIXES (9 findings incl. skippable allergy gate; S5 ledger reconciliation + clamp sign) -&gt; re-review PASS; 14 screens; Written 2026-09-15; S1/S2/S5/S9/S12 + recipe detail + states + legend/undo/who-did-what</t>
   </si>
   <si>
     <t>M3-E0-T2</t>
@@ -431,7 +428,7 @@
     <t>Check arithmetic; no token drift from prototype</t>
   </si>
   <si>
-    <t>Queued (after M3-E0-T1) - D-018a</t>
+    <t>In progress - dispatched 2026-09-16</t>
   </si>
   <si>
     <t>Output docs/design/tokens.md ready for the typed token module in M3</t>
@@ -1014,7 +1011,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67E6F0A1-0DCD-40C3-A117-E39AF7BCACDB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A54E7857-F83E-4422-831B-7C0F547CB7ED}">
   <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1639,18 +1636,18 @@
         <v>116</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>55</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>111</v>
@@ -1659,7 +1656,7 @@
         <v>112</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>17</v>
@@ -1668,16 +1665,16 @@
         <v>18</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I16" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>102</v>
@@ -1686,12 +1683,12 @@
         <v>55</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>111</v>
@@ -1700,7 +1697,7 @@
         <v>112</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>17</v>
@@ -1709,376 +1706,378 @@
         <v>18</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>18</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>110</v>
       </c>
       <c r="K17" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="M17" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>134</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F18" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="H18" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="J18" s="2" t="s">
+      <c r="K18" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>139</v>
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>143</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F19" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="I19" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>149</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G20" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>154</v>
-      </c>
       <c r="J20" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>158</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G21" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="H21" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I21" s="2" t="s">
+      <c r="J21" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="J21" s="2" t="s">
-        <v>161</v>
-      </c>
       <c r="K21" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>164</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>165</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G22" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I22" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="H22" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I22" s="2" t="s">
+      <c r="J22" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="J22" s="2" t="s">
-        <v>168</v>
-      </c>
       <c r="K22" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C23" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>171</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>172</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G23" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I23" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="H23" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I23" s="2" t="s">
+      <c r="J23" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="J23" s="2" t="s">
-        <v>175</v>
-      </c>
       <c r="K23" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G24" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I24" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="H24" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>181</v>
-      </c>
       <c r="J24" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C25" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>184</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>185</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G25" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I25" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="H25" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>187</v>
-      </c>
       <c r="J25" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>190</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G26" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I26" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="H26" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>192</v>
-      </c>
       <c r="J26" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L26" s="2"/>
       <c r="M26" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M26" xr:uid="{67E6F0A1-0DCD-40C3-A117-E39AF7BCACDB}"/>
+  <autoFilter ref="A1:M26" xr:uid="{A54E7857-F83E-4422-831B-7C0F547CB7ED}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M3-E0-T3 - review record (PASS after fixes); D-018a queue complete, engineering stopped for the PO/Dean session; token-darkening call added to the decision brief (A12)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3583944-EC0D-4A5A-88B7-86C37381DCD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C7E8A8B2-C673-4A36-942E-5F1EE4F77E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{31410C2C-C827-48E9-B149-314833D2161E}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{07316F56-BCB7-434D-98D2-8CC44DAF3C86}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="192">
   <si>
     <t>ID</t>
   </si>
@@ -428,10 +428,7 @@
     <t>Check arithmetic; no token drift from prototype</t>
   </si>
   <si>
-    <t>In progress - dispatched 2026-09-16</t>
-  </si>
-  <si>
-    <t>Output docs/design/tokens.md ready for the typed token module in M3</t>
+    <t>Review: PASS WITH FIXES (5 uncovered contrast pairs) -&gt; re-review PASS; 40 pairs; 16 FAILs w/ PROPOSED fixes (PO call); D-018a queue COMPLETE - stopped. Output docs/design/tokens.md ready for the typed token module in M3</t>
   </si>
   <si>
     <t>M2</t>
@@ -1011,7 +1008,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A54E7857-F83E-4422-831B-7C0F547CB7ED}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E843669C-351B-48FF-80DE-CF0B14ADFB6A}">
   <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1718,366 +1715,366 @@
         <v>110</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>69</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F18" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="H18" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="I18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="J18" s="2" t="s">
+      <c r="K18" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>138</v>
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>142</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F19" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="I19" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>148</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>151</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G20" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>153</v>
-      </c>
       <c r="J20" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>156</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>157</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G21" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="H21" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="I21" s="2" t="s">
+      <c r="J21" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="J21" s="2" t="s">
-        <v>160</v>
-      </c>
       <c r="K21" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>164</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G22" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I22" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="H22" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="I22" s="2" t="s">
+      <c r="J22" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="J22" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="K22" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C23" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>171</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G23" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I23" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="H23" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="I23" s="2" t="s">
+      <c r="J23" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="J23" s="2" t="s">
-        <v>174</v>
-      </c>
       <c r="K23" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>177</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>178</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G24" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I24" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="H24" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>180</v>
-      </c>
       <c r="J24" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C25" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>183</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>184</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G25" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I25" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="H25" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>186</v>
-      </c>
       <c r="J25" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>189</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G26" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I26" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="H26" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>191</v>
-      </c>
       <c r="J26" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L26" s="2"/>
       <c r="M26" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M26" xr:uid="{A54E7857-F83E-4422-831B-7C0F547CB7ED}"/>
+  <autoFilter ref="A1:M26" xr:uid="{E843669C-351B-48FF-80DE-CF0B14ADFB6A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(tracker): regenerate BACKLOG_TRACKER.xlsx from CSV (M2-T1..T3, M3-T1..T4c rows)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andy\OneDrive\006_Smart Kitchen App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C7E8A8B2-C673-4A36-942E-5F1EE4F77E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DEA0DE4A-1DC3-42A7-BD08-190717038837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{07316F56-BCB7-434D-98D2-8CC44DAF3C86}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="38700" windowHeight="15345" xr2:uid="{F7533918-6AB0-4865-A90E-79322388B4DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$35</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="260">
   <si>
     <t>ID</t>
   </si>
@@ -618,6 +618,210 @@
   </si>
   <si>
     <t>Pre-launch legal gates R-3/R-4/R-5</t>
+  </si>
+  <si>
+    <t>M3-T1</t>
+  </si>
+  <si>
+    <t>M3 build (D-023)</t>
+  </si>
+  <si>
+    <t>Expo app scaffold, D-021 tokens, five-slot tab shell with Menu placeholder, fixture ApiClient</t>
+  </si>
+  <si>
+    <t>Tooling and shell inside an established token system; no product logic</t>
+  </si>
+  <si>
+    <t>No rule-23 risk; token numbers, rule-11 dependencies, CI integration</t>
+  </si>
+  <si>
+    <t>M0-T1; M0-T2 (done)</t>
+  </si>
+  <si>
+    <t>Done - accepted &amp; merged 2026-09-22 (11e79fb)</t>
+  </si>
+  <si>
+    <t>Review: PASS WITH FIXES (relative-path domain-boundary bypass) -&gt; fix -&gt; PASS</t>
+  </si>
+  <si>
+    <t>M2-T1</t>
+  </si>
+  <si>
+    <t>M2 (D-022 stubbed identity)</t>
+  </si>
+  <si>
+    <t>Identity port with fixture adapter, default-deny authorization, tenant-scoped sessions, GET /v1/inventory/items, redacted logging</t>
+  </si>
+  <si>
+    <t>Household authorization and tenancy isolation (rule 23)</t>
+  </si>
+  <si>
+    <t>Adversarial: reach another household through every layer</t>
+  </si>
+  <si>
+    <t>M1-T2; M1-T9; M1-T11 (done)</t>
+  </si>
+  <si>
+    <t>Done - accepted &amp; merged 2026-09-22 (079bfc1)</t>
+  </si>
+  <si>
+    <t>Opus worker / Opus reviewer / architect pass</t>
+  </si>
+  <si>
+    <t>Review: PASS WITH FIXES (compiled API could not start; 500 logging; production guard denylist) -&gt; fixes -&gt; architect F8 clean-state lint -&gt; fix -&gt; PASS</t>
+  </si>
+  <si>
+    <t>M3-T2</t>
+  </si>
+  <si>
+    <t>Onboarding S1 account + household and S2 allergies with the explicit-none gate, first-run routing guard, onboarding state behind the client port</t>
+  </si>
+  <si>
+    <t>Screens inside the shell; a small gating state machine</t>
+  </si>
+  <si>
+    <t>Allergy gate is safety copy (P5, D-017)</t>
+  </si>
+  <si>
+    <t>M3-T1 (done)</t>
+  </si>
+  <si>
+    <t>Done - accepted &amp; merged 2026-09-22 (2f44fb6)</t>
+  </si>
+  <si>
+    <t>Sonnet worker / Opus reviewer</t>
+  </si>
+  <si>
+    <t>Review: PASS WITH FIXES (copy scan blind to JSX; deep links bypassed the gate; Node globals leak; copy) -&gt; fixes -&gt; re-review found a stale-read redirect bounce -&gt; fix -&gt; PASS</t>
+  </si>
+  <si>
+    <t>M3-T3</t>
+  </si>
+  <si>
+    <t>Inventory list S4 and item detail S5 with ledger history, HttpApiClient read, correction/removal/undo behind the port</t>
+  </si>
+  <si>
+    <t>Display of exact quantities and a fixture ledger</t>
+  </si>
+  <si>
+    <t>Ledger semantics on screen (rule 23)</t>
+  </si>
+  <si>
+    <t>M3-T1; M3-T2; M2-T1 (done)</t>
+  </si>
+  <si>
+    <t>Done - accepted &amp; merged 2026-09-22 (b41b809)</t>
+  </si>
+  <si>
+    <t>Review: PASS WITH FIXES (non-discriminating float test; unreachable empty state; failed save reported success) -&gt; fixes -&gt; PASS</t>
+  </si>
+  <si>
+    <t>M2-T2</t>
+  </si>
+  <si>
+    <t>Inventory write endpoints (FEFO allocation, idempotent replay, undo), GET item detail, dev seed command</t>
+  </si>
+  <si>
+    <t>Ledger writes, idempotency, concurrency, tenancy over writes (rule 23)</t>
+  </si>
+  <si>
+    <t>Adversarial: double-apply, cross-household, forged actor, partial commit, seed isolation</t>
+  </si>
+  <si>
+    <t>M2-T1; M1-T8; M1-T9; M1-T11; M3-T3 (done)</t>
+  </si>
+  <si>
+    <t>Done - accepted &amp; merged 2026-09-22 (994d829)</t>
+  </si>
+  <si>
+    <t>Review: PASS WITH FIXES (AJV stripped unknown fields; negative target minted a fake clamp) -&gt; fixes -&gt; PASS; 1559 tests with DB</t>
+  </si>
+  <si>
+    <t>M3-T4a</t>
+  </si>
+  <si>
+    <t>Client plumbing: writes/detail/undo wired to M2-T2, UUIDv7 idempotency keys (expo-crypto), copy-deck §8 error strings, component test library, global toast host</t>
+  </si>
+  <si>
+    <t>Wiring an existing port to existing endpoints</t>
+  </si>
+  <si>
+    <t>Key reuse on retry, error strings, component tests</t>
+  </si>
+  <si>
+    <t>M2-T2; M3-T3 (done)</t>
+  </si>
+  <si>
+    <t>Done - accepted &amp; merged 2026-09-22 (0122ced)</t>
+  </si>
+  <si>
+    <t>Review: PASS (no code fixes); architect ruling adopted expo-crypto over a Math.random fallback -&gt; PASS</t>
+  </si>
+  <si>
+    <t>M3-T4b</t>
+  </si>
+  <si>
+    <t>Add food: S6 hub, S7 expo-camera scan, S8 confirm with the allergen row from engine-generated screening fixtures, S9 manual add, fixture lookup and createItem</t>
+  </si>
+  <si>
+    <t>Screens plus one Expo module; no safety computation in the client</t>
+  </si>
+  <si>
+    <t>Scan-sheet allergen row is safety copy (P5, D-017, SR-1/SR-2)</t>
+  </si>
+  <si>
+    <t>M3-T4a (done)</t>
+  </si>
+  <si>
+    <t>Done - accepted &amp; merged 2026-09-23 (62ef687)</t>
+  </si>
+  <si>
+    <t>Review: FAIL (hand-derived verdict ALLOWED where the engine says ALLOWED_WITH_UNKNOWNS) -&gt; engine-generated fixtures with drift test, per-line rendering, 18 fixes -&gt; PASS WITH FIXES (float guard, loading gate) -&gt; PASS</t>
+  </si>
+  <si>
+    <t>M2-T3</t>
+  </si>
+  <si>
+    <t>Household create, join by code (migration 0008), members, item creation over the ledger</t>
+  </si>
+  <si>
+    <t>Membership is the tenancy boundary (rule 23)</t>
+  </si>
+  <si>
+    <t>Adversarial: code brute force, join twice, create in a foreign household, replay</t>
+  </si>
+  <si>
+    <t>M2-T1; M2-T2; M3-T4b (done)</t>
+  </si>
+  <si>
+    <t>Written 2026-09-23 - held for PO usage reset</t>
+  </si>
+  <si>
+    <t>M2-T4 (restrictions storage, product lookup endpoint, server-side screening) outlined, gated on A3</t>
+  </si>
+  <si>
+    <t>M3-T4c</t>
+  </si>
+  <si>
+    <t>Web target for desk review, Expo start hygiene (EXPO_NO_TYPESCRIPT_SETUP), SDK-aligned safe-area-context and screens</t>
+  </si>
+  <si>
+    <t>Tooling and dependency alignment; no domain logic</t>
+  </si>
+  <si>
+    <t>Verify clean tree after expo start and every screen on web from an empty build state</t>
+  </si>
+  <si>
+    <t>M3-T4b (done)</t>
+  </si>
+  <si>
+    <t>Written 2026-09-23 - dispatched</t>
+  </si>
+  <si>
+    <t>Sonnet worker</t>
+  </si>
+  <si>
+    <t>Triggered by Andy's first local run: expo start rewrote tsconfig.json (breaks typecheck and format), w failed without react-native-web</t>
   </si>
 </sst>
 </file>
@@ -1008,8 +1212,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E843669C-351B-48FF-80DE-CF0B14ADFB6A}">
-  <dimension ref="A1:M26"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13FF31D9-E4CC-4B78-8318-324EE71126E2}">
+  <dimension ref="A1:M35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -1021,7 +1225,7 @@
     <col min="7" max="7" width="60.7109375" customWidth="1"/>
     <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="60.7109375" customWidth="1"/>
-    <col min="10" max="10" width="39.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="39.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="60.7109375" customWidth="1"/>
     <col min="12" max="12" width="50.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="60.7109375" customWidth="1"/>
@@ -2073,8 +2277,377 @@
         <v>191</v>
       </c>
     </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="L27" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M27" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="L28" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="L29" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="M29" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="M30" s="2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="L32" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="M33" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M34" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="M35" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M26" xr:uid="{E843669C-351B-48FF-80DE-CF0B14ADFB6A}"/>
+  <autoFilter ref="A1:M35" xr:uid="{13FF31D9-E4CC-4B78-8318-324EE71126E2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(tracker): regenerate xlsx (M3-T4c done)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andy\OneDrive\006_Smart Kitchen App\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DEA0DE4A-1DC3-42A7-BD08-190717038837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0FB9D02A-2CAC-4860-A693-A6181F7276B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="38700" windowHeight="15345" xr2:uid="{F7533918-6AB0-4865-A90E-79322388B4DF}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="38700" windowHeight="15345" xr2:uid="{A391AF6B-41DE-4387-B698-A50F306BDCB8}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="259">
   <si>
     <t>ID</t>
   </si>
@@ -815,10 +815,7 @@
     <t>M3-T4b (done)</t>
   </si>
   <si>
-    <t>Written 2026-09-23 - dispatched</t>
-  </si>
-  <si>
-    <t>Sonnet worker</t>
+    <t>Done - accepted &amp; merged 2026-09-24 (8620bb7); PO browser walk owed</t>
   </si>
   <si>
     <t>Triggered by Andy's first local run: expo start rewrote tsconfig.json (breaks typecheck and format), w failed without react-native-web</t>
@@ -1212,7 +1209,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13FF31D9-E4CC-4B78-8318-324EE71126E2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EF0619C-4D70-483E-BC49-7AED29C0B2C6}">
   <dimension ref="A1:M35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2640,14 +2637,14 @@
         <v>257</v>
       </c>
       <c r="L35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M35" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="M35" s="2" t="s">
-        <v>259</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M35" xr:uid="{13FF31D9-E4CC-4B78-8318-324EE71126E2}"/>
+  <autoFilter ref="A1:M35" xr:uid="{4EF0619C-4D70-483E-BC49-7AED29C0B2C6}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M2-T3 - review record (PASS WITH FIXES then PASS, architect code pass), ARCHITECTURE §7 and data-model §2 join codes and membership doors, copy-deck §8 household refusals, DECISIONS OQ-E2 note + OQ-E3 join code expiry + OQ-E4 create while a member, BACKLOG follow-ups and scope widening, STATUS, tracker (script path moved to D:)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0FB9D02A-2CAC-4860-A693-A6181F7276B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{65F6AE1D-5775-4888-879A-97D20FC5F986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="38700" windowHeight="15345" xr2:uid="{A391AF6B-41DE-4387-B698-A50F306BDCB8}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="38700" windowHeight="15345" xr2:uid="{B1382857-A53E-4EB3-BCFC-D3704F99E29A}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$36</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="268">
   <si>
     <t>ID</t>
   </si>
@@ -794,7 +794,7 @@
     <t>M2-T1; M2-T2; M3-T4b (done)</t>
   </si>
   <si>
-    <t>Written 2026-09-23 - held for PO usage reset</t>
+    <t>Done - accepted &amp; merged 2026-09-29 (dcdd3cd)</t>
   </si>
   <si>
     <t>M2-T4 (restrictions storage, product lookup endpoint, server-side screening) outlined, gated on A3</t>
@@ -819,6 +819,33 @@
   </si>
   <si>
     <t>Triggered by Andy's first local run: expo start rewrote tsconfig.json (breaks typecheck and format), w failed without react-native-web</t>
+  </si>
+  <si>
+    <t>M3-T5</t>
+  </si>
+  <si>
+    <t>M3 Client (Expo)</t>
+  </si>
+  <si>
+    <t>M3 build (D-023 locked screens)</t>
+  </si>
+  <si>
+    <t>Shopping list S11: gap rows with origin chips, check-off with the close-the-loop prompt, in-session offline queue (fixture-backed)</t>
+  </si>
+  <si>
+    <t>Screen inside the established shell and tokens; fixture data behind the port; no gap math in the client</t>
+  </si>
+  <si>
+    <t>Queued check-off replay is idempotency semantics (rule 23) and the loop Add writes a ledger row</t>
+  </si>
+  <si>
+    <t>M3-T4c (done)</t>
+  </si>
+  <si>
+    <t>In review - round 1 FAIL (queue lost on unmount; stale replay; double Add); fix round in progress</t>
+  </si>
+  <si>
+    <t>Runs in parallel with M2-T3; D-024 rows 10 and 13 become a follow-up ticket if accepted</t>
   </si>
 </sst>
 </file>
@@ -1209,8 +1236,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EF0619C-4D70-483E-BC49-7AED29C0B2C6}">
-  <dimension ref="A1:M35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CA71DDC-8215-4341-8E5D-89604C1612B8}">
+  <dimension ref="A1:M36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -2643,8 +2670,49 @@
         <v>258</v>
       </c>
     </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M35" xr:uid="{4EF0619C-4D70-483E-BC49-7AED29C0B2C6}"/>
+  <autoFilter ref="A1:M36" xr:uid="{1CA71DDC-8215-4341-8E5D-89604C1612B8}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M2-T3a - hotfix review record appended, BACKLOG ticket record and follow-up, STATUS lesson (DB tickets wait for the CI run before the acceptance docs commit), tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{65F6AE1D-5775-4888-879A-97D20FC5F986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C704E23-8D1A-4BC3-8278-DB5A3DEFA0AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="38700" windowHeight="15345" xr2:uid="{B1382857-A53E-4EB3-BCFC-D3704F99E29A}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="38700" windowHeight="15345" xr2:uid="{1E8E5D25-AEF1-4E68-91B7-9C02677BD82A}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$37</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="275">
   <si>
     <t>ID</t>
   </si>
@@ -846,6 +846,27 @@
   </si>
   <si>
     <t>Runs in parallel with M2-T3; D-024 rows 10 and 13 become a follow-up ticket if accepted</t>
+  </si>
+  <si>
+    <t>M2-T3a</t>
+  </si>
+  <si>
+    <t>Hotfix: join-code rotation clock (transaction-start now() tripped the revoked-after-created check under concurrency in CI)</t>
+  </si>
+  <si>
+    <t>Tenancy-adjacent DB write found red on main by CI</t>
+  </si>
+  <si>
+    <t>Same reviewer re-check of a two-file diff</t>
+  </si>
+  <si>
+    <t>M2-T3 (done)</t>
+  </si>
+  <si>
+    <t>Done - accepted &amp; merged 2026-09-29 (3591bf8)</t>
+  </si>
+  <si>
+    <t>Deterministic two-connection reproduction added; clock_timestamp() for both stamps under the advisory lock</t>
   </si>
 </sst>
 </file>
@@ -1236,8 +1257,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CA71DDC-8215-4341-8E5D-89604C1612B8}">
-  <dimension ref="A1:M36"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{636EDE6F-7E24-47F5-BF09-7D1D5063A8D5}">
+  <dimension ref="A1:M37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -2711,8 +2732,49 @@
         <v>267</v>
       </c>
     </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M36" xr:uid="{1CA71DDC-8215-4341-8E5D-89604C1612B8}"/>
+  <autoFilter ref="A1:M37" xr:uid="{636EDE6F-7E24-47F5-BF09-7D1D5063A8D5}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M3-T5 - review record (FAIL, PASS WITH FIXES x2, PASS), copy-deck §7 S11 strings and §8 read fallback, ux-plan S11 loop-bar rule, BACKLOG DONE + follow-ups (M7 Add-once rule, connectivity signal, unit union, sufficient convention, persistence), STATUS, tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C704E23-8D1A-4BC3-8278-DB5A3DEFA0AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1EAD9ACC-6146-4C48-92E4-6A1E11337713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="38700" windowHeight="15345" xr2:uid="{1E8E5D25-AEF1-4E68-91B7-9C02677BD82A}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="38700" windowHeight="15345" xr2:uid="{CB9F1430-D07E-4793-99DC-38708F9410A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -842,7 +842,7 @@
     <t>M3-T4c (done)</t>
   </si>
   <si>
-    <t>In review - round 1 FAIL (queue lost on unmount; stale replay; double Add); fix round in progress</t>
+    <t>Done - accepted &amp; merged 2026-09-29 (dba4a7a)</t>
   </si>
   <si>
     <t>Runs in parallel with M2-T3; D-024 rows 10 and 13 become a follow-up ticket if accepted</t>
@@ -1257,7 +1257,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{636EDE6F-7E24-47F5-BF09-7D1D5063A8D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C46D28A6-28D1-4FE5-A0F4-1FA80A34953E}">
   <dimension ref="A1:M37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2774,7 +2774,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M37" xr:uid="{636EDE6F-7E24-47F5-BF09-7D1D5063A8D5}"/>
+  <autoFilter ref="A1:M37" xr:uid="{C46D28A6-28D1-4FE5-A0F4-1FA80A34953E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: D-025 live Open Food Facts lookup approved and unbundled from A3 (PO 2026-09-29); tickets M2-T4a (OFF adapter + GET /v1/products/{code} + NOT_RUN screening state) and M3-T4d (client wiring to the M2-T3 endpoints) written and dispatched; M3-T4e outlined; copy-deck §3.3 NOT_RUN row; ADR-006 partial-adoption note; STATUS; tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1EAD9ACC-6146-4C48-92E4-6A1E11337713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{89AA10D0-5094-45A4-9ADC-CDE81901C54A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="38700" windowHeight="15345" xr2:uid="{CB9F1430-D07E-4793-99DC-38708F9410A4}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{ABB18FB8-F655-4028-9773-A39BF7FA7B4C}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$39</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="289">
   <si>
     <t>ID</t>
   </si>
@@ -867,6 +867,48 @@
   </si>
   <si>
     <t>Deterministic two-connection reproduction added; clock_timestamp() for both stamps under the advisory lock</t>
+  </si>
+  <si>
+    <t>M2-T4a</t>
+  </si>
+  <si>
+    <t>Product lookup over Open Food Facts (server-side), GET /v1/products/{code}, explicit not-run screening state on the scan sheet</t>
+  </si>
+  <si>
+    <t>Data boundary the scan sheet trusts: provenance tiers</t>
+  </si>
+  <si>
+    <t>allergen tag mapping</t>
+  </si>
+  <si>
+    <t>external service failure modes</t>
+  </si>
+  <si>
+    <t>Adversarial: Known Fact leakage</t>
+  </si>
+  <si>
+    <t>absence-from-missing-data</t>
+  </si>
+  <si>
+    <t>429 as not-found</t>
+  </si>
+  <si>
+    <t>M3-T4d</t>
+  </si>
+  <si>
+    <t>Client wiring to the M2-T3 endpoints: create household, join by code, household read, item creation over HTTP</t>
+  </si>
+  <si>
+    <t>Client plumbing against existing endpoints (M3-T4a pattern)</t>
+  </si>
+  <si>
+    <t>Idempotent creation over the network and the create-or-join flow that picks the household</t>
+  </si>
+  <si>
+    <t>Dispatched 2026-09-29</t>
+  </si>
+  <si>
+    <t>Runs in parallel with M2-T4a; lookupProduct wiring is M3-T4e</t>
   </si>
 </sst>
 </file>
@@ -1257,8 +1299,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C46D28A6-28D1-4FE5-A0F4-1FA80A34953E}">
-  <dimension ref="A1:M37"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AE6EC60-BD4D-497A-B2FC-DD6788E718F1}">
+  <dimension ref="A1:M39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -1268,7 +1310,7 @@
     <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="60.7109375" customWidth="1"/>
-    <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="60.7109375" customWidth="1"/>
     <col min="10" max="10" width="39.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="60.7109375" customWidth="1"/>
@@ -2773,8 +2815,90 @@
         <v>274</v>
       </c>
     </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="L39" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M39" s="2" t="s">
+        <v>288</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M37" xr:uid="{C46D28A6-28D1-4FE5-A0F4-1FA80A34953E}"/>
+  <autoFilter ref="A1:M39" xr:uid="{4AE6EC60-BD4D-497A-B2FC-DD6788E718F1}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M2-T4a - review record (PASS WITH FIXES then PASS, architect code pass), ADR-006 Open Food Facts tier policy and R-4 note, copy-deck §3.3 label fields and §8 lookup refusals, BACKLOG rate-limit correction + follow-ups + M3-T4e written, STATUS, tracker; README curl example moves the fixture token into a variable (gitleaks curl-auth-header finding on 4af01c9); CONTRIBUTING secret-scanning note
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{89AA10D0-5094-45A4-9ADC-CDE81901C54A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A6E03A2-546E-46CD-AE4D-F7DFC6C328BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{ABB18FB8-F655-4028-9773-A39BF7FA7B4C}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{D6623B50-93C1-4D1A-9EFB-E1D1F8BDB0F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -1299,7 +1299,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AE6EC60-BD4D-497A-B2FC-DD6788E718F1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A307EA65-4134-4B40-A037-4A0C48C39EBD}">
   <dimension ref="A1:M39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2898,7 +2898,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M39" xr:uid="{4AE6EC60-BD4D-497A-B2FC-DD6788E718F1}"/>
+  <autoFilter ref="A1:M39" xr:uid="{A307EA65-4134-4B40-A037-4A0C48C39EBD}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: apply the M2-T4a acceptance edits the 01b48d1 message described (its doc script failed to parse): ADR-006 Open Food Facts tier policy and R-4 note, copy-deck §3.3 label fields and §8 lookup refusals, BACKLOG M2-T4a DONE + rate-limit correction + follow-ups + M3-T4e ticket written, STATUS, tracker CSV
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A6E03A2-546E-46CD-AE4D-F7DFC6C328BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{89E09FA4-6BF3-4B1F-9670-2CC665C85E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{D6623B50-93C1-4D1A-9EFB-E1D1F8BDB0F0}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{F43D2BDC-FCDB-439E-94D0-ABA228DEC4F1}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$40</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="297">
   <si>
     <t>ID</t>
   </si>
@@ -909,6 +909,30 @@
   </si>
   <si>
     <t>Runs in parallel with M2-T4a; lookupProduct wiring is M3-T4e</t>
+  </si>
+  <si>
+    <t>M3-T4e</t>
+  </si>
+  <si>
+    <t>lookupProduct over HTTP and the scan sheet on live Open Food Facts data: nutrition basis, quantity tier, lookup refusals, package units, held key on S8</t>
+  </si>
+  <si>
+    <t>Client wiring plus fully specified rendering rules; one small adapter rule</t>
+  </si>
+  <si>
+    <t>First time live Estimated data reaches the add path: tier upgrades</t>
+  </si>
+  <si>
+    <t>nutrition basis</t>
+  </si>
+  <si>
+    <t>message leaks</t>
+  </si>
+  <si>
+    <t>double Save</t>
+  </si>
+  <si>
+    <t>M2-T4a and M3-T4d (done)</t>
   </si>
 </sst>
 </file>
@@ -1299,8 +1323,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A307EA65-4134-4B40-A037-4A0C48C39EBD}">
-  <dimension ref="A1:M39"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C59875F-E9E6-413E-8285-527C408E6962}">
+  <dimension ref="A1:M40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -2897,8 +2921,49 @@
         <v>288</v>
       </c>
     </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>296</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M39" xr:uid="{A307EA65-4134-4B40-A037-4A0C48C39EBD}"/>
+  <autoFilter ref="A1:M40" xr:uid="{1C59875F-E9E6-413E-8285-527C408E6962}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M3-T4d - review record (PASS WITH FIXES x2 then PASS, two approved scope widenings), copy-deck §11 HTTP-only post-create string and failed-read strings, BACKLOG premise corrected + DONE + follow-ups, STATUS (M3-T4e dispatched), tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{89E09FA4-6BF3-4B1F-9670-2CC665C85E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A4A3E37-64D8-4FBA-A116-5FFD0ED1C6FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{F43D2BDC-FCDB-439E-94D0-ABA228DEC4F1}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{DFBBA85F-FDE0-4269-8B8F-E1F7C1ACD29A}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -905,7 +905,7 @@
     <t>Idempotent creation over the network and the create-or-join flow that picks the household</t>
   </si>
   <si>
-    <t>Dispatched 2026-09-29</t>
+    <t>Done - accepted &amp; merged 2026-09-29 (8d1217b)</t>
   </si>
   <si>
     <t>Runs in parallel with M2-T4a; lookupProduct wiring is M3-T4e</t>
@@ -1323,7 +1323,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C59875F-E9E6-413E-8285-527C408E6962}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6183FD79-6536-4A72-913C-B3DF02DD5FF1}">
   <dimension ref="A1:M40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2963,7 +2963,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M40" xr:uid="{1C59875F-E9E6-413E-8285-527C408E6962}"/>
+  <autoFilter ref="A1:M40" xr:uid="{6183FD79-6536-4A72-913C-B3DF02DD5FF1}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M3-T4e - review record (PASS WITH FIXES then PASS, 21 mutations caught), copy-deck §7 S8 live-data strings (nutrition basis, not on file, package-of, caption, quantity source, toast tier word), ADR-006 absent nutrition_data_per rule, BACKLOG DONE + objective (e) amended + follow-ups (CI export flags, S8 read fallback, PER_100ML), STATUS (scan flow end to end; fridge test owed), README stale lines, tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A4A3E37-64D8-4FBA-A116-5FFD0ED1C6FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1286706-C595-441F-B448-3602A28030CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{DFBBA85F-FDE0-4269-8B8F-E1F7C1ACD29A}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{AFD0E8E7-2099-4547-B042-8DE14F6D3521}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -1323,7 +1323,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6183FD79-6536-4A72-913C-B3DF02DD5FF1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19F6CB72-37CF-47A8-9A82-A4923F1E68B6}">
   <dimension ref="A1:M40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2963,7 +2963,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M40" xr:uid="{6183FD79-6536-4A72-913C-B3DF02DD5FF1}"/>
+  <autoFilter ref="A1:M40" xr:uid="{19F6CB72-37CF-47A8-9A82-A4923F1E68B6}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: batch A written (PO go 2026-09-29): tickets M3-T6 profile, M7-T1 shopping persistence and endpoints, R-6 FoodKeeper shelf-life research, M2-T4b lookup hardening, M9-T0 maintenance bundle 2, M9-D1 architecture docs pass; D-026 gluten tag mapping PROPOSED; STATUS (M3-T6, M7-T1, R-6 dispatched); tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1286706-C595-441F-B448-3602A28030CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BBCBE872-D960-4944-AA79-8A6F8742062B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{AFD0E8E7-2099-4547-B042-8DE14F6D3521}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="38700" windowHeight="15345" xr2:uid="{00E98124-3D72-4ABD-B96F-62426CBCC8CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="336">
   <si>
     <t>ID</t>
   </si>
@@ -933,6 +933,123 @@
   </si>
   <si>
     <t>M2-T4a and M3-T4d (done)</t>
+  </si>
+  <si>
+    <t>M3-T6</t>
+  </si>
+  <si>
+    <t>Profile and household (S12): members with per-member allergy edit, join code for the owner, sign-out</t>
+  </si>
+  <si>
+    <t>Screen reusing S2 components and existing endpoints</t>
+  </si>
+  <si>
+    <t>Allergy edit surface and an owner-only action</t>
+  </si>
+  <si>
+    <t>M3-T4d (done)</t>
+  </si>
+  <si>
+    <t>Dispatched 2026-09-29</t>
+  </si>
+  <si>
+    <t>Batch A</t>
+  </si>
+  <si>
+    <t>M7-T1</t>
+  </si>
+  <si>
+    <t>Shopping list persistence and endpoints: migration 0009, gap math on the server, check-off, add-to-inventory once per row, HTTP client wiring</t>
+  </si>
+  <si>
+    <t>Rule-7 gap math, a PURCHASE ledger write, once-per-row idempotency</t>
+  </si>
+  <si>
+    <t>Adversarial: double add, cross-household, gap drift, replay conflicts</t>
+  </si>
+  <si>
+    <t>M2-T3 and M3-T5 (done)</t>
+  </si>
+  <si>
+    <t>R-6</t>
+  </si>
+  <si>
+    <t>R (research)</t>
+  </si>
+  <si>
+    <t>Shelf-life data research: USDA FoodKeeper coverage, licence and the estimation rule (docs only)</t>
+  </si>
+  <si>
+    <t>Research</t>
+  </si>
+  <si>
+    <t>R-1 pattern: script, raw capture, findings</t>
+  </si>
+  <si>
+    <t>Licence and numbers reproduced</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>Batch A; no signup, no spend; feeds M8-T1</t>
+  </si>
+  <si>
+    <t>M2-T4b</t>
+  </si>
+  <si>
+    <t>Product lookup hardening: UPC-E, GTIN-14, English-name fallback, gluten tag mapping (D-026)</t>
+  </si>
+  <si>
+    <t>Contained adapter and validator changes</t>
+  </si>
+  <si>
+    <t>Allergen map and code expansion decide what a scan resolves to</t>
+  </si>
+  <si>
+    <t>M2-T4a and M3-T4e (done)</t>
+  </si>
+  <si>
+    <t>Written 2026-09-29; after M7-T1 and M3-T6 merge</t>
+  </si>
+  <si>
+    <t>M9-T0</t>
+  </si>
+  <si>
+    <t>M9 Hardening</t>
+  </si>
+  <si>
+    <t>Maintenance bundle 2 (accepted follow-ups from the 2026-09-29 reviews)</t>
+  </si>
+  <si>
+    <t>Small fully specified items</t>
+  </si>
+  <si>
+    <t>Nothing weakened</t>
+  </si>
+  <si>
+    <t>M2-T3a and M3-T4e (done)</t>
+  </si>
+  <si>
+    <t>M9-D1</t>
+  </si>
+  <si>
+    <t>Architecture documentation pass (docs only)</t>
+  </si>
+  <si>
+    <t>Docs</t>
+  </si>
+  <si>
+    <t>architect</t>
+  </si>
+  <si>
+    <t>rule 15 housekeeping</t>
+  </si>
+  <si>
+    <t>batch A merges</t>
+  </si>
+  <si>
+    <t>Written 2026-09-29</t>
   </si>
 </sst>
 </file>
@@ -1323,15 +1440,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19F6CB72-37CF-47A8-9A82-A4923F1E68B6}">
-  <dimension ref="A1:M40"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D6E844B-C9BE-4FCE-8963-2650A90669C8}">
+  <dimension ref="A1:M46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="60.7109375" customWidth="1"/>
-    <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="60.7109375" customWidth="1"/>
     <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
@@ -2962,8 +3078,254 @@
         <v>296</v>
       </c>
     </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M43" s="2" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M44" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M45" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="M46" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M40" xr:uid="{19F6CB72-37CF-47A8-9A82-A4923F1E68B6}"/>
+  <autoFilter ref="A1:M46" xr:uid="{3D6E844B-C9BE-4FCE-8963-2650A90669C8}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: M9-D1 architecture documentation pass - ARCHITECTURE status and §2 shape as built, §3 table rows for the decided client, backend and database, §7 household isolation names the real RLS; ADR-004 target line (built on the stubbed port); ADR-010 progress note (in-session shopping queue built, persistence is M7-T3); ADR README statuses; no decision changed
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BBCBE872-D960-4944-AA79-8A6F8742062B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D9B061F-A58F-4579-8878-7CFFEB72B0D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="38700" windowHeight="15345" xr2:uid="{00E98124-3D72-4ABD-B96F-62426CBCC8CB}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{B4E685B7-AA83-40DB-BDC9-9A13AF690C05}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -1049,7 +1049,7 @@
     <t>batch A merges</t>
   </si>
   <si>
-    <t>Written 2026-09-29</t>
+    <t>Done 2026-09-30 (architect)</t>
   </si>
 </sst>
 </file>
@@ -1440,7 +1440,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D6E844B-C9BE-4FCE-8963-2650A90669C8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17D48338-2356-4A8D-97DD-37F799023AB3}">
   <dimension ref="A1:M46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3325,7 +3325,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M46" xr:uid="{3D6E844B-C9BE-4FCE-8963-2650A90669C8}"/>
+  <autoFilter ref="A1:M46" xr:uid="{17D48338-2356-4A8D-97DD-37F799023AB3}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M7-T1 - review record (PASS WITH FIXES then PASS, architect code pass), data-model §2 shopping_rows and shopping_row_writes with the read-time gap rule and §6 replay note, BACKLOG DONE + rulings + follow-ups (M7-T2, M7-T3, generation bump, boolean bodies, member-leave policy), STATUS, tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D9B061F-A58F-4579-8878-7CFFEB72B0D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{149FBEFE-3317-4256-A13A-2A9478BD91D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{B4E685B7-AA83-40DB-BDC9-9A13AF690C05}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{2FA5E7F7-FE5B-49CA-9FE5-E13A9CB40FC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="337">
   <si>
     <t>ID</t>
   </si>
@@ -969,6 +969,9 @@
   </si>
   <si>
     <t>M2-T3 and M3-T5 (done)</t>
+  </si>
+  <si>
+    <t>Done - accepted &amp; merged 2026-09-30 (01fca8a)</t>
   </si>
   <si>
     <t>R-6</t>
@@ -1440,7 +1443,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17D48338-2356-4A8D-97DD-37F799023AB3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BE6C13-3664-4D8F-9DC6-EEE368B33D76}">
   <dimension ref="A1:M46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3151,7 +3154,7 @@
         <v>308</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="L42" s="2" t="s">
         <v>131</v>
@@ -3162,34 +3165,34 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>182</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>18</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="K43" s="2" t="s">
         <v>302</v>
@@ -3198,12 +3201,12 @@
         <v>131</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>155</v>
@@ -3212,7 +3215,7 @@
         <v>154</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>17</v>
@@ -3221,19 +3224,19 @@
         <v>18</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="L44" s="2" t="s">
         <v>131</v>
@@ -3244,16 +3247,16 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>186</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>17</v>
@@ -3262,19 +3265,19 @@
         <v>18</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>18</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="L45" s="2" t="s">
         <v>131</v>
@@ -3285,25 +3288,25 @@
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>186</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>131</v>
@@ -3312,20 +3315,20 @@
         <v>131</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="M46" s="2" t="s">
         <v>303</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M46" xr:uid="{17D48338-2356-4A8D-97DD-37F799023AB3}"/>
+  <autoFilter ref="A1:M46" xr:uid="{73BE6C13-3664-4D8F-9DC6-EEE368B33D76}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M3-T6 - review record (PASS WITH FIXES x2 then PASS), copy-deck §7 S12 and §11 S1 note, BACKLOG DONE + objective (c) history corrected + follow-ups, STATUS (README rewrite was the PO's agent; BUG-001, BUG-002, M9-T0 dispatched), tracker; the M2-T4a review record missed at its acceptance; PO bug tickets BUG-001 and BUG-002 committed as OPEN records; D-027 browser-origin allowlist PROPOSED; README cd lines (PO)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{149FBEFE-3317-4256-A13A-2A9478BD91D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F703919-CAE6-4308-9498-038E0256051B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{2FA5E7F7-FE5B-49CA-9FE5-E13A9CB40FC0}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="38700" windowHeight="15345" xr2:uid="{BB1D1CA0-EB6A-44BA-AD61-7FB8EFA7F831}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="339">
   <si>
     <t>ID</t>
   </si>
@@ -950,51 +950,54 @@
     <t>M3-T4d (done)</t>
   </si>
   <si>
+    <t>Done - accepted &amp; merged 2026-09-30 (74371f1)</t>
+  </si>
+  <si>
+    <t>Batch A</t>
+  </si>
+  <si>
+    <t>M7-T1</t>
+  </si>
+  <si>
+    <t>Shopping list persistence and endpoints: migration 0009, gap math on the server, check-off, add-to-inventory once per row, HTTP client wiring</t>
+  </si>
+  <si>
+    <t>Rule-7 gap math, a PURCHASE ledger write, once-per-row idempotency</t>
+  </si>
+  <si>
+    <t>Adversarial: double add, cross-household, gap drift, replay conflicts</t>
+  </si>
+  <si>
+    <t>M2-T3 and M3-T5 (done)</t>
+  </si>
+  <si>
+    <t>Done - accepted &amp; merged 2026-09-30 (01fca8a)</t>
+  </si>
+  <si>
+    <t>R-6</t>
+  </si>
+  <si>
+    <t>R (research)</t>
+  </si>
+  <si>
+    <t>Shelf-life data research: USDA FoodKeeper coverage, licence and the estimation rule (docs only)</t>
+  </si>
+  <si>
+    <t>Research</t>
+  </si>
+  <si>
+    <t>R-1 pattern: script, raw capture, findings</t>
+  </si>
+  <si>
+    <t>Licence and numbers reproduced</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
     <t>Dispatched 2026-09-29</t>
   </si>
   <si>
-    <t>Batch A</t>
-  </si>
-  <si>
-    <t>M7-T1</t>
-  </si>
-  <si>
-    <t>Shopping list persistence and endpoints: migration 0009, gap math on the server, check-off, add-to-inventory once per row, HTTP client wiring</t>
-  </si>
-  <si>
-    <t>Rule-7 gap math, a PURCHASE ledger write, once-per-row idempotency</t>
-  </si>
-  <si>
-    <t>Adversarial: double add, cross-household, gap drift, replay conflicts</t>
-  </si>
-  <si>
-    <t>M2-T3 and M3-T5 (done)</t>
-  </si>
-  <si>
-    <t>Done - accepted &amp; merged 2026-09-30 (01fca8a)</t>
-  </si>
-  <si>
-    <t>R-6</t>
-  </si>
-  <si>
-    <t>R (research)</t>
-  </si>
-  <si>
-    <t>Shelf-life data research: USDA FoodKeeper coverage, licence and the estimation rule (docs only)</t>
-  </si>
-  <si>
-    <t>Research</t>
-  </si>
-  <si>
-    <t>R-1 pattern: script, raw capture, findings</t>
-  </si>
-  <si>
-    <t>Licence and numbers reproduced</t>
-  </si>
-  <si>
-    <t>none</t>
-  </si>
-  <si>
     <t>Batch A; no signup, no spend; feeds M8-T1</t>
   </si>
   <si>
@@ -1013,25 +1016,28 @@
     <t>M2-T4a and M3-T4e (done)</t>
   </si>
   <si>
+    <t>Dispatched 2026-09-30</t>
+  </si>
+  <si>
+    <t>M9-T0</t>
+  </si>
+  <si>
+    <t>M9 Hardening</t>
+  </si>
+  <si>
+    <t>Maintenance bundle 2 (accepted follow-ups from the 2026-09-29 reviews)</t>
+  </si>
+  <si>
+    <t>Small fully specified items</t>
+  </si>
+  <si>
+    <t>Nothing weakened</t>
+  </si>
+  <si>
+    <t>M2-T3a and M3-T4e (done)</t>
+  </si>
+  <si>
     <t>Written 2026-09-29; after M7-T1 and M3-T6 merge</t>
-  </si>
-  <si>
-    <t>M9-T0</t>
-  </si>
-  <si>
-    <t>M9 Hardening</t>
-  </si>
-  <si>
-    <t>Maintenance bundle 2 (accepted follow-ups from the 2026-09-29 reviews)</t>
-  </si>
-  <si>
-    <t>Small fully specified items</t>
-  </si>
-  <si>
-    <t>Nothing weakened</t>
-  </si>
-  <si>
-    <t>M2-T3a and M3-T4e (done)</t>
   </si>
   <si>
     <t>M9-D1</t>
@@ -1443,7 +1449,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BE6C13-3664-4D8F-9DC6-EEE368B33D76}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4DD05CF-4B1B-4204-A052-8847FB9435EA}">
   <dimension ref="A1:M46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3195,18 +3201,18 @@
         <v>316</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>302</v>
+        <v>317</v>
       </c>
       <c r="L43" s="2" t="s">
         <v>131</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>155</v>
@@ -3215,7 +3221,7 @@
         <v>154</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>17</v>
@@ -3224,19 +3230,19 @@
         <v>18</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="L44" s="2" t="s">
         <v>131</v>
@@ -3247,16 +3253,16 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>186</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>17</v>
@@ -3265,19 +3271,19 @@
         <v>18</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>18</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="L45" s="2" t="s">
         <v>131</v>
@@ -3288,25 +3294,25 @@
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>186</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>131</v>
@@ -3315,20 +3321,20 @@
         <v>131</v>
       </c>
       <c r="J46" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="L46" s="2" t="s">
         <v>335</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="L46" s="2" t="s">
-        <v>333</v>
       </c>
       <c r="M46" s="2" t="s">
         <v>303</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M46" xr:uid="{73BE6C13-3664-4D8F-9DC6-EEE368B33D76}"/>
+  <autoFilter ref="A1:M46" xr:uid="{B4DD05CF-4B1B-4204-A052-8847FB9435EA}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M9-T0 - review record (PASS WITH FIXES then PASS), BACKLOG DONE + rulings + the two flakes on record, STATUS, tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F703919-CAE6-4308-9498-038E0256051B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1CD59ADC-A065-45FC-9765-AAA4FF95B40C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="38700" windowHeight="15345" xr2:uid="{BB1D1CA0-EB6A-44BA-AD61-7FB8EFA7F831}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{A7C57EE4-5134-476F-B0F0-70E7847818C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -1037,7 +1037,7 @@
     <t>M2-T3a and M3-T4e (done)</t>
   </si>
   <si>
-    <t>Written 2026-09-29; after M7-T1 and M3-T6 merge</t>
+    <t>Done - accepted &amp; merged 2026-10-01 (86965b6)</t>
   </si>
   <si>
     <t>M9-D1</t>
@@ -1449,7 +1449,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4DD05CF-4B1B-4204-A052-8847FB9435EA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74D45E76-07FF-4CE9-9DB5-9780F667E853}">
   <dimension ref="A1:M46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3334,7 +3334,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M46" xr:uid="{B4DD05CF-4B1B-4204-A052-8847FB9435EA}"/>
+  <autoFilter ref="A1:M46" xr:uid="{74D45E76-07FF-4CE9-9DB5-9780F667E853}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M2-T4b - review record (FAIL on D-026 then PASS), ADR-006 code handling (UPC-E precedence, 58% collision, GS1-8 RCN prefixes), D-026 built as amended, BACKLOG DONE + follow-ups (symbology priority raised, GTIN14 at the port, leading-1 test gap, identity-mapping decision for M2-T4, OFF usage form, request budget), STATUS, tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1CD59ADC-A065-45FC-9765-AAA4FF95B40C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1E72D26-28C7-4062-BB92-807EB3C9B613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{A7C57EE4-5134-476F-B0F0-70E7847818C2}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{3C8315B9-8FCB-4EE0-83A6-1D781CA251AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -1016,7 +1016,7 @@
     <t>M2-T4a and M3-T4e (done)</t>
   </si>
   <si>
-    <t>Dispatched 2026-09-30</t>
+    <t>Done - accepted &amp; merged 2026-10-01 (a622495)</t>
   </si>
   <si>
     <t>M9-T0</t>
@@ -1449,7 +1449,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74D45E76-07FF-4CE9-9DB5-9780F667E853}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1137798C-0BFA-4AC8-9ADB-8E2E10328D54}">
   <dimension ref="A1:M46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3334,7 +3334,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M46" xr:uid="{74D45E76-07FF-4CE9-9DB5-9780F667E853}"/>
+  <autoFilter ref="A1:M46" xr:uid="{1137798C-0BFA-4AC8-9ADB-8E2E10328D54}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept BUG-002 - review record (PASS WITH FIXES then PASS), bug ticket FIXED, ARCHITECTURE 7.11 browser-origin rule, D-027 built as proposed (PO ratifies), BACKLOG follow-ups (deploy checklist, expose-headers, allow-headers), STATUS (batch A status, owed PO lines, R-6 blocked on the FoodKeeper download), tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1E72D26-28C7-4062-BB92-807EB3C9B613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BC652D1-E067-45E3-93E0-5D4B1A5F60BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{3C8315B9-8FCB-4EE0-83A6-1D781CA251AA}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{489B9C05-22DA-4C55-912F-AEFC21C393BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$47</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="348">
   <si>
     <t>ID</t>
   </si>
@@ -1059,6 +1059,33 @@
   </si>
   <si>
     <t>Done 2026-09-30 (architect)</t>
+  </si>
+  <si>
+    <t>BUG-002</t>
+  </si>
+  <si>
+    <t>Bugs (PO device and browser tests)</t>
+  </si>
+  <si>
+    <t>API sends no CORS headers, web real mode blocked; fixed by the SK_CORS_ORIGINS allowlist (D-027)</t>
+  </si>
+  <si>
+    <t>Bug</t>
+  </si>
+  <si>
+    <t>Security boundary (browser origins)</t>
+  </si>
+  <si>
+    <t>Adversarial: leak with no allowlist</t>
+  </si>
+  <si>
+    <t>exact match</t>
+  </si>
+  <si>
+    <t>hook order</t>
+  </si>
+  <si>
+    <t>guard</t>
   </si>
 </sst>
 </file>
@@ -1449,8 +1476,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1137798C-0BFA-4AC8-9ADB-8E2E10328D54}">
-  <dimension ref="A1:M46"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D47CFAC-9581-4A0C-B6EA-80DE26553049}">
+  <dimension ref="A1:M47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -3333,8 +3360,49 @@
         <v>303</v>
       </c>
     </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="L47" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="M47" s="2" t="s">
+        <v>316</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M46" xr:uid="{1137798C-0BFA-4AC8-9ADB-8E2E10328D54}"/>
+  <autoFilter ref="A1:M47" xr:uid="{3D47CFAC-9581-4A0C-B6EA-80DE26553049}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept BUG-001 - review record (PASS WITH FIXES then PASS), bug ticket FIXED with the bisect and the fix, M3-T4d review amendment (navigator rule: never unmount after first mount), BACKLOG follow-ups (smoke script at acceptance, eslint block for scripts, inert for overlays, gate-covered rule for side-effectful screens, shared camera stand-in, long-read spinner, device-pass additions), STATUS (Android re-run owed, next 3 actions), tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BC652D1-E067-45E3-93E0-5D4B1A5F60BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{70E4F0CD-FB92-4D19-8C87-2A16BD691A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{489B9C05-22DA-4C55-912F-AEFC21C393BB}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{CDD53CBC-D5D7-4323-BFB0-3CD147CE25D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$48</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="355">
   <si>
     <t>ID</t>
   </si>
@@ -1086,6 +1086,27 @@
   </si>
   <si>
     <t>guard</t>
+  </si>
+  <si>
+    <t>BUG-001</t>
+  </si>
+  <si>
+    <t>S2 Continue crashes with Maximum update depth exceeded (Android and web); root layout unmounted the navigator mid-navigation</t>
+  </si>
+  <si>
+    <t>Onboarding gate; allergy-gate bypass is the risk</t>
+  </si>
+  <si>
+    <t>Adversarial: bypass under the cover</t>
+  </si>
+  <si>
+    <t>redirect semantics</t>
+  </si>
+  <si>
+    <t>stale read</t>
+  </si>
+  <si>
+    <t>failed read</t>
   </si>
 </sst>
 </file>
@@ -1476,8 +1497,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D47CFAC-9581-4A0C-B6EA-80DE26553049}">
-  <dimension ref="A1:M47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27212034-EC93-452F-8421-B4E73E28E006}">
+  <dimension ref="A1:M48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -3401,8 +3422,49 @@
         <v>316</v>
       </c>
     </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="M48" s="2" t="s">
+        <v>316</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M47" xr:uid="{3D47CFAC-9581-4A0C-B6EA-80DE26553049}"/>
+  <autoFilter ref="A1:M48" xr:uid="{27212034-EC93-452F-8421-B4E73E28E006}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(tracker): regenerate the workbook from the CSV (BUG-003, BUG-004, M3-T7, M2-T5, M2-T6 rows; the file was locked by Excel during the day's acceptances)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{70E4F0CD-FB92-4D19-8C87-2A16BD691A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{00EB1DE5-BEF1-4D50-808D-1D28E7644616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{CDD53CBC-D5D7-4323-BFB0-3CD147CE25D4}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="24885" windowHeight="15345" xr2:uid="{6F3160EF-E955-4289-B491-FE35BEB53C28}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$53</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="388">
   <si>
     <t>ID</t>
   </si>
@@ -1107,6 +1107,105 @@
   </si>
   <si>
     <t>failed read</t>
+  </si>
+  <si>
+    <t>BUG-003</t>
+  </si>
+  <si>
+    <t>Scan sheet under the Android navigation bar, camera panel too tall, list screens under the floating tab bar</t>
+  </si>
+  <si>
+    <t>Layout only</t>
+  </si>
+  <si>
+    <t>Insets and clearance pinned per screen</t>
+  </si>
+  <si>
+    <t>Fixed 2026-10-01 (88881e1)</t>
+  </si>
+  <si>
+    <t>Reported by Andy 2026-10-01</t>
+  </si>
+  <si>
+    <t>BUG-004</t>
+  </si>
+  <si>
+    <t>Confirm on an AI proposal throws an uncaught rejection over the API (crash guard)</t>
+  </si>
+  <si>
+    <t>Error path only</t>
+  </si>
+  <si>
+    <t>Rejection handled, no unhandled promise</t>
+  </si>
+  <si>
+    <t>Fixed 2026-10-01 (523bbf2)</t>
+  </si>
+  <si>
+    <t>M2-T5</t>
+  </si>
+  <si>
+    <t>M2 API</t>
+  </si>
+  <si>
+    <t>Inventory</t>
+  </si>
+  <si>
+    <t>Confirm an AI proposal over the API: endpoint, provenance confirmation, client wiring</t>
+  </si>
+  <si>
+    <t>Feature</t>
+  </si>
+  <si>
+    <t>AI output crossing into domain state; idempotency; tenancy</t>
+  </si>
+  <si>
+    <t>Adversarial: cross-household, double confirm, non-proposal</t>
+  </si>
+  <si>
+    <t>BUG-004 (client part)</t>
+  </si>
+  <si>
+    <t>Dispatched 2026-10-01</t>
+  </si>
+  <si>
+    <t>From the 2026-10-01 device test</t>
+  </si>
+  <si>
+    <t>M3-T7</t>
+  </si>
+  <si>
+    <t>Typed quantities on the S5 correction card and an editable package size on the S8 scan sheet</t>
+  </si>
+  <si>
+    <t>Inventory arithmetic through free text</t>
+  </si>
+  <si>
+    <t>Exact micros, tier flip pinned</t>
+  </si>
+  <si>
+    <t>Written 2026-10-01, queued</t>
+  </si>
+  <si>
+    <t>Andy: 125 g vs 248 g, 500 taps</t>
+  </si>
+  <si>
+    <t>M2-T6</t>
+  </si>
+  <si>
+    <t>Move an item between locations (D-024 row 1): migration 0010, endpoint, S5 action</t>
+  </si>
+  <si>
+    <t>Migration next to inventory history; household write</t>
+  </si>
+  <si>
+    <t>Ledger untouched by a move, idempotent</t>
+  </si>
+  <si>
+    <t>M3-T7 (S5 part)</t>
+  </si>
+  <si>
+    <t>D-024 row 1 approved by Andy 2026-10-01</t>
   </si>
 </sst>
 </file>
@@ -1497,8 +1596,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27212034-EC93-452F-8421-B4E73E28E006}">
-  <dimension ref="A1:M48"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A50364-6853-4F2B-8319-754F5A0024C4}">
+  <dimension ref="A1:M53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -3463,8 +3562,213 @@
         <v>316</v>
       </c>
     </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="L49" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M49" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="M50" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="L51" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M51" s="2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="L52" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M52" s="2" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M53" s="2" t="s">
+        <v>387</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M48" xr:uid="{27212034-EC93-452F-8421-B4E73E28E006}"/>
+  <autoFilter ref="A1:M53" xr:uid="{89A50364-6853-4F2B-8319-754F5A0024C4}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M2-T5 and M3-T7 - review records (M2-T5: conflict then PASS WITH FIXES then PASS; M3-T7: PASS WITH FIXES x3 then PASS), BACKLOG DONE + follow-ups (typed confirmation state, startup migration check, remove-member FK, lot label and quantity source on the wire, locale decimal, range check), D-028 built as proposed, ARCHITECTURE 7.4 confirm route, data-model confirmations table and the ledger UNIQUE, copy-deck 4 confirmed source and 7 S5/S8 typed fields, STATUS (migrate the practice DB with db:migrate before the API; M2-T6 dispatched), tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{00EB1DE5-BEF1-4D50-808D-1D28E7644616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5788E533-9D52-4B48-8F00-496F8010D15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="24885" windowHeight="15345" xr2:uid="{6F3160EF-E955-4289-B491-FE35BEB53C28}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{2FB5A669-749C-4191-BF26-85200CEA7774}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="389">
   <si>
     <t>ID</t>
   </si>
@@ -1166,7 +1166,7 @@
     <t>BUG-004 (client part)</t>
   </si>
   <si>
-    <t>Dispatched 2026-10-01</t>
+    <t>Done 2026-10-01 (dab68f1)</t>
   </si>
   <si>
     <t>From the 2026-10-01 device test</t>
@@ -1184,25 +1184,28 @@
     <t>Exact micros, tier flip pinned</t>
   </si>
   <si>
+    <t>Done 2026-10-02 (7b73c0d)</t>
+  </si>
+  <si>
+    <t>Andy: 125 g vs 248 g, 500 taps</t>
+  </si>
+  <si>
+    <t>M2-T6</t>
+  </si>
+  <si>
+    <t>Move an item between locations (D-024 row 1): migration 0010, endpoint, S5 action</t>
+  </si>
+  <si>
+    <t>Migration next to inventory history; household write</t>
+  </si>
+  <si>
+    <t>Ledger untouched by a move, idempotent</t>
+  </si>
+  <si>
+    <t>M3-T7 (S5 part)</t>
+  </si>
+  <si>
     <t>Written 2026-10-01, queued</t>
-  </si>
-  <si>
-    <t>Andy: 125 g vs 248 g, 500 taps</t>
-  </si>
-  <si>
-    <t>M2-T6</t>
-  </si>
-  <si>
-    <t>Move an item between locations (D-024 row 1): migration 0010, endpoint, S5 action</t>
-  </si>
-  <si>
-    <t>Migration next to inventory history; household write</t>
-  </si>
-  <si>
-    <t>Ledger untouched by a move, idempotent</t>
-  </si>
-  <si>
-    <t>M3-T7 (S5 part)</t>
   </si>
   <si>
     <t>D-024 row 1 approved by Andy 2026-10-01</t>
@@ -1596,7 +1599,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A50364-6853-4F2B-8319-754F5A0024C4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60C43A91-CA55-4A73-AE40-31825D16FBD1}">
   <dimension ref="A1:M53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3758,17 +3761,17 @@
         <v>386</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="L53" s="2" t="s">
         <v>131</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M53" xr:uid="{89A50364-6853-4F2B-8319-754F5A0024C4}"/>
+  <autoFilter ref="A1:M53" xr:uid="{60C43A91-CA55-4A73-AE40-31825D16FBD1}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M2-T6 - review record (PASS WITH FIXES then PASS by a fresh reviewer), BACKLOG DONE + follow-ups (deploy order 0010 and 0011, history clocks and move tie-break, typed SAME_LOCATION, remove-member FK, S4 Other group, focus refetch), D-024 row 1 built with the open expiry question for the PO, ARCHITECTURE 7.4 move route, data-model moves table and storage_location rule, copy-deck 4 no chip on a move and 7 S5 Move to states, STATUS (db:migrate again for 0011; re-test list), tracker
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5788E533-9D52-4B48-8F00-496F8010D15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D135F66D-4012-4A53-98A9-BE0D9594D1E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{2FB5A669-749C-4191-BF26-85200CEA7774}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{C1283A58-25BE-430C-9525-41E93477E1A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -1205,7 +1205,7 @@
     <t>M3-T7 (S5 part)</t>
   </si>
   <si>
-    <t>Written 2026-10-01, queued</t>
+    <t>Done 2026-10-02 (ada4455)</t>
   </si>
   <si>
     <t>D-024 row 1 approved by Andy 2026-10-01</t>
@@ -1599,7 +1599,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60C43A91-CA55-4A73-AE40-31825D16FBD1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A44A1F2A-F12D-40B5-A94C-DFD994B3A9F2}">
   <dimension ref="A1:M53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3771,7 +3771,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M53" xr:uid="{60C43A91-CA55-4A73-AE40-31825D16FBD1}"/>
+  <autoFilter ref="A1:M53" xr:uid="{A44A1F2A-F12D-40B5-A94C-DFD994B3A9F2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept BUG-005 (review PASS, Sonnet, lean brief) - review record, bug ticket FIXED, CONTRIBUTING rule on agent worktrees and Metro, BACKLOG follow-ups, STATUS, tracker; chore(deps): audit exception for GHSA-vfj7-8cjw-p6xm (braces, no patched version, dev tooling only; the CI audit step went red on f8a5b51 the hour it was published)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D135F66D-4012-4A53-98A9-BE0D9594D1E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E3ACE37-FA30-4E17-B3E1-6E452123D5BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{C1283A58-25BE-430C-9525-41E93477E1A1}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{0FEED96C-9B46-4642-A025-A95EFB965D7D}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$54</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="395">
   <si>
     <t>ID</t>
   </si>
@@ -1209,6 +1209,24 @@
   </si>
   <si>
     <t>D-024 row 1 approved by Andy 2026-10-01</t>
+  </si>
+  <si>
+    <t>BUG-005</t>
+  </si>
+  <si>
+    <t>Metro served the bundle before its index was ready: 34 agent worktrees in the watch folder; block list fix</t>
+  </si>
+  <si>
+    <t>Tooling config</t>
+  </si>
+  <si>
+    <t>Config test and smoke</t>
+  </si>
+  <si>
+    <t>Fixed 2026-10-03 (f8a5b51)</t>
+  </si>
+  <si>
+    <t>Reported by Andy 2026-10-02; cause: architect's unpruned worktrees</t>
   </si>
 </sst>
 </file>
@@ -1599,8 +1617,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A44A1F2A-F12D-40B5-A94C-DFD994B3A9F2}">
-  <dimension ref="A1:M53"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C1B94C-6791-4A5D-8CF7-62CDC20D1BDE}">
+  <dimension ref="A1:M54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -3770,8 +3788,49 @@
         <v>388</v>
       </c>
     </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="L54" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M54" s="2" t="s">
+        <v>394</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M53" xr:uid="{A44A1F2A-F12D-40B5-A94C-DFD994B3A9F2}"/>
+  <autoFilter ref="A1:M54" xr:uid="{33C1B94C-6791-4A5D-8CF7-62CDC20D1BDE}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M3-T8 (review PASS, Sonnet) - review record, ticket archived, BUG-001 follow-ups marked done, STATUS, tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E3ACE37-FA30-4E17-B3E1-6E452123D5BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5D8CAC9-B19E-411F-8BD6-FC243DA48D5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15345" xr2:uid="{0FEED96C-9B46-4642-A025-A95EFB965D7D}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{CE71538A-F401-4592-9B5D-0D59E8AFAF23}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$57</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="416">
   <si>
     <t>ID</t>
   </si>
@@ -1227,6 +1227,69 @@
   </si>
   <si>
     <t>Reported by Andy 2026-10-02; cause: architect's unpruned worktrees</t>
+  </si>
+  <si>
+    <t>M2-T4c</t>
+  </si>
+  <si>
+    <t>Product lookup</t>
+  </si>
+  <si>
+    <t>Send the scanned symbology with the lookup; GTIN14 port normalisation</t>
+  </si>
+  <si>
+    <t>Contract and route parsing</t>
+  </si>
+  <si>
+    <t>Hint only narrows</t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>M2-T4b follow-up (priority raised)</t>
+  </si>
+  <si>
+    <t>M3-T8</t>
+  </si>
+  <si>
+    <t>Test infrastructure</t>
+  </si>
+  <si>
+    <t>Lint block for app scripts; shared camera stand-in for the S7 gate tests</t>
+  </si>
+  <si>
+    <t>Chore</t>
+  </si>
+  <si>
+    <t>Tooling and tests</t>
+  </si>
+  <si>
+    <t>No assertion weakened</t>
+  </si>
+  <si>
+    <t>Done 2026-10-06 (0c4db1f)</t>
+  </si>
+  <si>
+    <t>BUG-001 follow-ups</t>
+  </si>
+  <si>
+    <t>M2-T7</t>
+  </si>
+  <si>
+    <t>Lot label and quantity origin on item create</t>
+  </si>
+  <si>
+    <t>Small contract and service change</t>
+  </si>
+  <si>
+    <t>Idempotent replay comparison</t>
+  </si>
+  <si>
+    <t>Ready</t>
+  </si>
+  <si>
+    <t>M3-T7 follow-up</t>
   </si>
 </sst>
 </file>
@@ -1617,8 +1680,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C1B94C-6791-4A5D-8CF7-62CDC20D1BDE}">
-  <dimension ref="A1:M54"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{616264DD-59D7-4184-B3B6-24BC87A301F9}">
+  <dimension ref="A1:M57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -3829,8 +3892,131 @@
         <v>394</v>
       </c>
     </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="L55" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M55" s="2" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M56" s="2" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="L57" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="M57" s="2" t="s">
+        <v>415</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M54" xr:uid="{33C1B94C-6791-4A5D-8CF7-62CDC20D1BDE}"/>
+  <autoFilter ref="A1:M57" xr:uid="{616264DD-59D7-4184-B3B6-24BC87A301F9}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M2-T4c (review PASS WITH FIXES then PASS, Sonnet) - review record, ticket archived, system-context product lookup route with the type hint and the iOS ean13 mapping, follow-ups (device pass for type strings, typed 8-digit overlap), STATUS, tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5D8CAC9-B19E-411F-8BD6-FC243DA48D5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{382CCB3B-8C8C-427C-8303-416F487092E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{CE71538A-F401-4592-9B5D-0D59E8AFAF23}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{A1FC2F56-7A5E-416B-9FB5-9732076F256A}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -1244,49 +1244,49 @@
     <t>Hint only narrows</t>
   </si>
   <si>
+    <t>Done 2026-10-06 (c82a642)</t>
+  </si>
+  <si>
+    <t>M2-T4b follow-up (priority raised)</t>
+  </si>
+  <si>
+    <t>M3-T8</t>
+  </si>
+  <si>
+    <t>Test infrastructure</t>
+  </si>
+  <si>
+    <t>Lint block for app scripts; shared camera stand-in for the S7 gate tests</t>
+  </si>
+  <si>
+    <t>Chore</t>
+  </si>
+  <si>
+    <t>Tooling and tests</t>
+  </si>
+  <si>
+    <t>No assertion weakened</t>
+  </si>
+  <si>
+    <t>Done 2026-10-06 (0c4db1f)</t>
+  </si>
+  <si>
+    <t>BUG-001 follow-ups</t>
+  </si>
+  <si>
+    <t>M2-T7</t>
+  </si>
+  <si>
+    <t>Lot label and quantity origin on item create</t>
+  </si>
+  <si>
+    <t>Small contract and service change</t>
+  </si>
+  <si>
+    <t>Idempotent replay comparison</t>
+  </si>
+  <si>
     <t>In progress</t>
-  </si>
-  <si>
-    <t>M2-T4b follow-up (priority raised)</t>
-  </si>
-  <si>
-    <t>M3-T8</t>
-  </si>
-  <si>
-    <t>Test infrastructure</t>
-  </si>
-  <si>
-    <t>Lint block for app scripts; shared camera stand-in for the S7 gate tests</t>
-  </si>
-  <si>
-    <t>Chore</t>
-  </si>
-  <si>
-    <t>Tooling and tests</t>
-  </si>
-  <si>
-    <t>No assertion weakened</t>
-  </si>
-  <si>
-    <t>Done 2026-10-06 (0c4db1f)</t>
-  </si>
-  <si>
-    <t>BUG-001 follow-ups</t>
-  </si>
-  <si>
-    <t>M2-T7</t>
-  </si>
-  <si>
-    <t>Lot label and quantity origin on item create</t>
-  </si>
-  <si>
-    <t>Small contract and service change</t>
-  </si>
-  <si>
-    <t>Idempotent replay comparison</t>
-  </si>
-  <si>
-    <t>Ready</t>
   </si>
   <si>
     <t>M3-T7 follow-up</t>
@@ -1680,7 +1680,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{616264DD-59D7-4184-B3B6-24BC87A301F9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B66595A0-72C3-4A99-8E2A-96552BE81D34}">
   <dimension ref="A1:M57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4016,7 +4016,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M57" xr:uid="{616264DD-59D7-4184-B3B6-24BC87A301F9}"/>
+  <autoFilter ref="A1:M57" xr:uid="{B66595A0-72C3-4A99-8E2A-96552BE81D34}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M2-T7 (review PASS, Opus, architect code pass clean) - review record, ticket archived, data-model 4 server-assigned create sources and the lot label replay rule, follow-ups (surrogate validation on create text fields), STATUS next actions, tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{382CCB3B-8C8C-427C-8303-416F487092E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E4F0023D-09F7-4297-853E-4EF65D6A3AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{A1FC2F56-7A5E-416B-9FB5-9732076F256A}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{0F3DFFBD-5E1B-4238-91C2-7E475878BD4E}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -1286,7 +1286,7 @@
     <t>Idempotent replay comparison</t>
   </si>
   <si>
-    <t>In progress</t>
+    <t>Done 2026-10-06 (9e41b98)</t>
   </si>
   <si>
     <t>M3-T7 follow-up</t>
@@ -1680,7 +1680,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B66595A0-72C3-4A99-8E2A-96552BE81D34}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46CAB5D0-DD2F-49FB-AFEA-6E98DB518A23}">
   <dimension ref="A1:M57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4016,7 +4016,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M57" xr:uid="{B66595A0-72C3-4A99-8E2A-96552BE81D34}"/>
+  <autoFilter ref="A1:M57" xr:uid="{46CAB5D0-DD2F-49FB-AFEA-6E98DB518A23}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M9-T1 (PASS), M9-T2, M3-T11 and M3-T12 (PASS WITH FIXES then PASS, Sonnet) - review records, tickets archived, copy-deck S5 tomorrow line, follow-ups (printed best-by stored as UTC midnight, vitest dist, override removal), tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E4F0023D-09F7-4297-853E-4EF65D6A3AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{42696C09-BDFD-40F3-990E-6C4F34A957F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{0F3DFFBD-5E1B-4238-91C2-7E475878BD4E}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{27DD5107-9878-42E7-9D82-4749B6B52550}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$66</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="469">
   <si>
     <t>ID</t>
   </si>
@@ -431,6 +431,27 @@
     <t>Review: PASS WITH FIXES (5 uncovered contrast pairs) -&gt; re-review PASS; 40 pairs; 16 FAILs w/ PROPOSED fixes (PO call); D-018a queue COMPLETE - stopped. Output docs/design/tokens.md ready for the typed token module in M3</t>
   </si>
   <si>
+    <t>M3-E0-T4</t>
+  </si>
+  <si>
+    <t>Prototype v5: unknown-allergen commit moment, one consistent household, a11y remedies (docs only)</t>
+  </si>
+  <si>
+    <t>HTML/CSS prototype work inside the token system</t>
+  </si>
+  <si>
+    <t>Allergen copy at the commit moment (rule 9 / rule 23)</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>In progress - dispatched 2026-10-07</t>
+  </si>
+  <si>
+    <t>From the impeccable critique of v4 (24/40); PO picked the three P1s; PO sees v5 before acceptance</t>
+  </si>
+  <si>
     <t>M2</t>
   </si>
   <si>
@@ -992,9 +1013,6 @@
     <t>Licence and numbers reproduced</t>
   </si>
   <si>
-    <t>none</t>
-  </si>
-  <si>
     <t>Dispatched 2026-09-29</t>
   </si>
   <si>
@@ -1290,6 +1308,147 @@
   </si>
   <si>
     <t>M3-T7 follow-up</t>
+  </si>
+  <si>
+    <t>M3-T9</t>
+  </si>
+  <si>
+    <t>A passed best-by reads expired (D-030), S4 and S5</t>
+  </si>
+  <si>
+    <t>Display-only helper and two screens</t>
+  </si>
+  <si>
+    <t>Not rule-23; provenance honesty of strings</t>
+  </si>
+  <si>
+    <t>Done 2026-10-07 (e944025)</t>
+  </si>
+  <si>
+    <t>Review PASS; follow-up: tomorrow reads use today</t>
+  </si>
+  <si>
+    <t>BUG-007</t>
+  </si>
+  <si>
+    <t>Bugs</t>
+  </si>
+  <si>
+    <t>Home header avatar clipped under the status bar</t>
+  </si>
+  <si>
+    <t>Small layout fix</t>
+  </si>
+  <si>
+    <t>Not rule-23</t>
+  </si>
+  <si>
+    <t>Done 2026-10-07 (82a03a0)</t>
+  </si>
+  <si>
+    <t>Review PASS; follow-up: top inset on every screen</t>
+  </si>
+  <si>
+    <t>BUG-006</t>
+  </si>
+  <si>
+    <t>M7 Shopping</t>
+  </si>
+  <si>
+    <t>A checked shopping row shows 0 lb</t>
+  </si>
+  <si>
+    <t>Shopping gap read and PURCHASE path (rule 23)</t>
+  </si>
+  <si>
+    <t>Rule 23</t>
+  </si>
+  <si>
+    <t>Done 2026-10-07 (c047edf)</t>
+  </si>
+  <si>
+    <t>Review PASS; architect code pass clean; PO question on two row display edge cases</t>
+  </si>
+  <si>
+    <t>M2-T8</t>
+  </si>
+  <si>
+    <t>Count units take whole numbers only (D-029), client and server</t>
+  </si>
+  <si>
+    <t>Inventory arithmetic on every write path (rule 23)</t>
+  </si>
+  <si>
+    <t>Done 2026-10-07 (f640e2c)</t>
+  </si>
+  <si>
+    <t>Review PASS WITH FIXES then PASS (Sonnet re-check); architect code pass clean</t>
+  </si>
+  <si>
+    <t>M9-T1</t>
+  </si>
+  <si>
+    <t>Maintenance</t>
+  </si>
+  <si>
+    <t>CI red: pnpm audit on shell-quote and source-map-js</t>
+  </si>
+  <si>
+    <t>Transitive pins only</t>
+  </si>
+  <si>
+    <t>Tooling</t>
+  </si>
+  <si>
+    <t>Done 2026-10-07 (376f62b)</t>
+  </si>
+  <si>
+    <t>Review PASS; follow-up: drop the overrides when parents pull patched ranges</t>
+  </si>
+  <si>
+    <t>M9-T2</t>
+  </si>
+  <si>
+    <t>COUNT unit aliases published from contracts with a consistency test</t>
+  </si>
+  <si>
+    <t>List move plus a test</t>
+  </si>
+  <si>
+    <t>Done 2026-10-07 (8948abb)</t>
+  </si>
+  <si>
+    <t>Review PASS WITH FIXES (format) then PASS</t>
+  </si>
+  <si>
+    <t>M3-T11</t>
+  </si>
+  <si>
+    <t>A best-by one day out reads tomorrow; calendar-day counts</t>
+  </si>
+  <si>
+    <t>Display wording</t>
+  </si>
+  <si>
+    <t>Done 2026-10-07 (84af14b)</t>
+  </si>
+  <si>
+    <t>Sent back once (rolling 24h); review PASS WITH FIXES (format) then PASS; follow-up: printed best-by stored as UTC midnight</t>
+  </si>
+  <si>
+    <t>M3-T12</t>
+  </si>
+  <si>
+    <t>One typed client ApiError; COUNT_NOT_WHOLE through ledgerErrorMessage</t>
+  </si>
+  <si>
+    <t>Client refactor</t>
+  </si>
+  <si>
+    <t>Done 2026-10-07 (d23a3c6)</t>
+  </si>
+  <si>
+    <t>Review PASS WITH FIXES (format) then PASS; follow-up: vitest dist and per-app run</t>
   </si>
 </sst>
 </file>
@@ -1680,14 +1839,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46CAB5D0-DD2F-49FB-AFEA-6E98DB518A23}">
-  <dimension ref="A1:M57"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F76AB62-8539-4782-B524-35130B55FA14}">
+  <dimension ref="A1:M66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="60.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="60.7109375" customWidth="1"/>
     <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
@@ -2400,151 +2560,153 @@
         <v>129</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="E18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="H18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="K18" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="I18" s="2" t="s">
+      <c r="L18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="M18" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F19" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="I19" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>147</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="G20" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="H20" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>152</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2" t="s">
@@ -2559,7 +2721,7 @@
         <v>162</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>163</v>
@@ -2568,13 +2730,13 @@
         <v>2</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>164</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>165</v>
@@ -2583,7 +2745,7 @@
         <v>166</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2" t="s">
@@ -2598,7 +2760,7 @@
         <v>169</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>170</v>
@@ -2607,13 +2769,13 @@
         <v>2</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>171</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>172</v>
@@ -2622,7 +2784,7 @@
         <v>173</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2" t="s">
@@ -2637,7 +2799,7 @@
         <v>176</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>177</v>
@@ -2646,239 +2808,237 @@
         <v>2</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>178</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>179</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>175</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
+      <c r="M25" s="2" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>2</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="L26" s="2"/>
-      <c r="M26" s="2" t="s">
-        <v>191</v>
-      </c>
+      <c r="M26" s="2"/>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="G27" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>18</v>
+        <v>140</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="K27" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="L27" s="2"/>
+      <c r="M27" s="2" t="s">
         <v>198</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>201</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>202</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="G28" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I28" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="H28" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="I28" s="2" t="s">
+      <c r="J28" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="J28" s="2" t="s">
+      <c r="K28" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="K28" s="2" t="s">
+      <c r="L28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M28" s="2" t="s">
         <v>206</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>209</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>210</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="G29" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I29" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="H29" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="I29" s="2" t="s">
+      <c r="J29" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="J29" s="2" t="s">
+      <c r="K29" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="K29" s="2" t="s">
+      <c r="L29" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="L29" s="2" t="s">
+      <c r="M29" s="2" t="s">
         <v>215</v>
-      </c>
-      <c r="M29" s="2" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>217</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>218</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>17</v>
@@ -2887,22 +3047,22 @@
         <v>18</v>
       </c>
       <c r="G30" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I30" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="H30" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="I30" s="2" t="s">
+      <c r="J30" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="J30" s="2" t="s">
+      <c r="K30" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="K30" s="2" t="s">
+      <c r="L30" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>215</v>
       </c>
       <c r="M30" s="2" t="s">
         <v>223</v>
@@ -2913,10 +3073,10 @@
         <v>224</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>225</v>
@@ -2925,7 +3085,7 @@
         <v>17</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>226</v>
@@ -2943,7 +3103,7 @@
         <v>229</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="M31" s="2" t="s">
         <v>230</v>
@@ -2954,10 +3114,10 @@
         <v>231</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>232</v>
@@ -2966,13 +3126,13 @@
         <v>17</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>233</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="I32" s="2" t="s">
         <v>234</v>
@@ -2984,7 +3144,7 @@
         <v>236</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>23</v>
+        <v>214</v>
       </c>
       <c r="M32" s="2" t="s">
         <v>237</v>
@@ -2995,10 +3155,10 @@
         <v>238</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>239</v>
@@ -3013,7 +3173,7 @@
         <v>240</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>241</v>
@@ -3025,7 +3185,7 @@
         <v>243</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>215</v>
+        <v>23</v>
       </c>
       <c r="M33" s="2" t="s">
         <v>244</v>
@@ -3036,10 +3196,10 @@
         <v>245</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>246</v>
@@ -3048,7 +3208,7 @@
         <v>17</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>247</v>
@@ -3066,7 +3226,7 @@
         <v>250</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>131</v>
+        <v>222</v>
       </c>
       <c r="M34" s="2" t="s">
         <v>251</v>
@@ -3077,10 +3237,10 @@
         <v>252</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>253</v>
@@ -3089,13 +3249,13 @@
         <v>17</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>254</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>255</v>
@@ -3107,7 +3267,7 @@
         <v>257</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>23</v>
+        <v>138</v>
       </c>
       <c r="M35" s="2" t="s">
         <v>258</v>
@@ -3118,13 +3278,13 @@
         <v>259</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>260</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>262</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>17</v>
@@ -3133,36 +3293,36 @@
         <v>18</v>
       </c>
       <c r="G36" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="J36" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="H36" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="I36" s="2" t="s">
+      <c r="K36" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="J36" s="2" t="s">
+      <c r="L36" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M36" s="2" t="s">
         <v>265</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>268</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>269</v>
@@ -3171,7 +3331,7 @@
         <v>17</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>270</v>
@@ -3189,7 +3349,7 @@
         <v>273</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="M37" s="2" t="s">
         <v>274</v>
@@ -3200,10 +3360,10 @@
         <v>275</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>276</v>
@@ -3218,77 +3378,77 @@
         <v>277</v>
       </c>
       <c r="H38" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I38" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="I38" s="2" t="s">
+      <c r="J38" s="2" t="s">
         <v>279</v>
-      </c>
-      <c r="J38" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="K38" s="2" t="s">
         <v>280</v>
       </c>
       <c r="L38" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M38" s="2" t="s">
         <v>281</v>
-      </c>
-      <c r="M38" s="2" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>283</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>284</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="G39" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="H39" s="2" t="s">
         <v>285</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>286</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>272</v>
+        <v>36</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>287</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>131</v>
+        <v>288</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>17</v>
@@ -3297,39 +3457,39 @@
         <v>18</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>293</v>
+        <v>279</v>
       </c>
       <c r="K40" s="2" t="s">
         <v>294</v>
       </c>
       <c r="L40" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M40" s="2" t="s">
         <v>295</v>
-      </c>
-      <c r="M40" s="2" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>297</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>298</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>17</v>
@@ -3338,22 +3498,22 @@
         <v>18</v>
       </c>
       <c r="G41" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I41" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="H41" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="I41" s="2" t="s">
+      <c r="J41" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="J41" s="2" t="s">
+      <c r="K41" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="K41" s="2" t="s">
+      <c r="L41" s="2" t="s">
         <v>302</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>131</v>
       </c>
       <c r="M41" s="2" t="s">
         <v>303</v>
@@ -3364,10 +3524,10 @@
         <v>304</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>176</v>
+        <v>267</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>175</v>
+        <v>268</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>305</v>
@@ -3376,7 +3536,7 @@
         <v>17</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>306</v>
@@ -3394,68 +3554,68 @@
         <v>309</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>182</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>311</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>312</v>
       </c>
       <c r="E43" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G43" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="F43" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G43" s="2" t="s">
+      <c r="H43" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I43" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="H43" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I43" s="2" t="s">
+      <c r="J43" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="J43" s="2" t="s">
+      <c r="K43" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="K43" s="2" t="s">
-        <v>317</v>
-      </c>
       <c r="L43" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="D44" s="2" t="s">
+      <c r="E44" s="2" t="s">
         <v>320</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>18</v>
@@ -3464,22 +3624,22 @@
         <v>321</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>322</v>
       </c>
       <c r="J44" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K44" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="K44" s="2" t="s">
+      <c r="L44" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M44" s="2" t="s">
         <v>324</v>
-      </c>
-      <c r="L44" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="M44" s="2" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
@@ -3487,13 +3647,13 @@
         <v>325</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>326</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>327</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>17</v>
@@ -3502,189 +3662,189 @@
         <v>18</v>
       </c>
       <c r="G45" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I45" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="H45" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I45" s="2" t="s">
+      <c r="J45" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="J45" s="2" t="s">
+      <c r="K45" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="K45" s="2" t="s">
-        <v>331</v>
-      </c>
       <c r="L45" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>326</v>
-      </c>
       <c r="C46" s="2" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>333</v>
       </c>
       <c r="E46" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G46" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="F46" s="2" t="s">
+      <c r="H46" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I46" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="J46" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="H46" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="I46" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="J46" s="2" t="s">
+      <c r="K46" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="K46" s="2" t="s">
-        <v>338</v>
-      </c>
       <c r="L46" s="2" t="s">
-        <v>335</v>
+        <v>138</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="B47" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="C47" s="2" t="s">
+      <c r="E47" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="D47" s="2" t="s">
+      <c r="F47" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="E47" s="2" t="s">
+      <c r="G47" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="F47" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G47" s="2" t="s">
+      <c r="H47" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="J47" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="H47" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="I47" s="2" t="s">
+      <c r="K47" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="J47" s="2" t="s">
-        <v>345</v>
-      </c>
-      <c r="K47" s="2" t="s">
-        <v>346</v>
-      </c>
       <c r="L47" s="2" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
       <c r="M47" s="2" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="E48" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="B48" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="D48" s="2" t="s">
+      <c r="F48" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G48" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="E48" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G48" s="2" t="s">
+      <c r="H48" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I48" s="2" t="s">
         <v>350</v>
       </c>
-      <c r="H48" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="I48" s="2" t="s">
+      <c r="J48" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="J48" s="2" t="s">
+      <c r="K48" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="K48" s="2" t="s">
+      <c r="L48" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="L48" s="2" t="s">
-        <v>354</v>
-      </c>
       <c r="M48" s="2" t="s">
-        <v>316</v>
+        <v>133</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="B49" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="D49" s="2" t="s">
+      <c r="E49" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G49" s="2" t="s">
         <v>356</v>
       </c>
-      <c r="E49" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G49" s="2" t="s">
+      <c r="H49" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I49" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="H49" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I49" s="2" t="s">
+      <c r="J49" s="2" t="s">
         <v>358</v>
-      </c>
-      <c r="J49" s="2" t="s">
-        <v>316</v>
       </c>
       <c r="K49" s="2" t="s">
         <v>359</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>131</v>
+        <v>360</v>
       </c>
       <c r="M49" s="2" t="s">
-        <v>360</v>
+        <v>133</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.25">
@@ -3692,16 +3852,16 @@
         <v>361</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>362</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>18</v>
@@ -3716,95 +3876,95 @@
         <v>364</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>316</v>
+        <v>133</v>
       </c>
       <c r="K50" s="2" t="s">
         <v>365</v>
       </c>
       <c r="L50" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M50" s="2" t="s">
         <v>366</v>
-      </c>
-      <c r="M50" s="2" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="L51" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="M51" s="2" t="s">
         <v>366</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="H51" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="I51" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="J51" s="2" t="s">
-        <v>373</v>
-      </c>
-      <c r="K51" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="L51" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="M51" s="2" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="E52" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="B52" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="D52" s="2" t="s">
+      <c r="F52" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G52" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="E52" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G52" s="2" t="s">
+      <c r="H52" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I52" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="H52" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="I52" s="2" t="s">
+      <c r="J52" s="2" t="s">
         <v>379</v>
-      </c>
-      <c r="J52" s="2" t="s">
-        <v>355</v>
       </c>
       <c r="K52" s="2" t="s">
         <v>380</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="M52" s="2" t="s">
         <v>381</v>
@@ -3815,16 +3975,16 @@
         <v>382</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>367</v>
+        <v>267</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>383</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>18</v>
@@ -3839,54 +3999,54 @@
         <v>385</v>
       </c>
       <c r="J53" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="K53" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="K53" s="2" t="s">
+      <c r="L53" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M53" s="2" t="s">
         <v>387</v>
-      </c>
-      <c r="L53" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="M53" s="2" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="D54" s="2" t="s">
+      <c r="E54" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G54" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="E54" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G54" s="2" t="s">
+      <c r="H54" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I54" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="H54" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I54" s="2" t="s">
+      <c r="J54" s="2" t="s">
         <v>392</v>
-      </c>
-      <c r="J54" s="2" t="s">
-        <v>316</v>
       </c>
       <c r="K54" s="2" t="s">
         <v>393</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="M54" s="2" t="s">
         <v>394</v>
@@ -3897,98 +4057,98 @@
         <v>395</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>367</v>
+        <v>267</v>
       </c>
       <c r="C55" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="D55" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="D55" s="2" t="s">
+      <c r="E55" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G55" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="E55" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G55" s="2" t="s">
+      <c r="H55" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I55" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="H55" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I55" s="2" t="s">
+      <c r="J55" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K55" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="J55" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="K55" s="2" t="s">
+      <c r="L55" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M55" s="2" t="s">
         <v>400</v>
-      </c>
-      <c r="L55" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="M55" s="2" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="C56" s="2" t="s">
+      <c r="D56" s="2" t="s">
         <v>403</v>
       </c>
-      <c r="D56" s="2" t="s">
+      <c r="E56" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G56" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="E56" s="2" t="s">
+      <c r="H56" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I56" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="F56" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G56" s="2" t="s">
+      <c r="J56" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K56" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="H56" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I56" s="2" t="s">
+      <c r="L56" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M56" s="2" t="s">
         <v>407</v>
-      </c>
-      <c r="J56" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="K56" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="L56" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="M56" s="2" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="B57" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="D57" s="2" t="s">
+      <c r="E57" s="2" t="s">
         <v>411</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>370</v>
       </c>
       <c r="F57" s="2" t="s">
         <v>18</v>
@@ -3997,26 +4157,395 @@
         <v>412</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="I57" s="2" t="s">
         <v>413</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>395</v>
+        <v>133</v>
       </c>
       <c r="K57" s="2" t="s">
         <v>414</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="M57" s="2" t="s">
         <v>415</v>
       </c>
     </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="L58" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M58" s="2" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="L59" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M59" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="L60" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M60" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="L61" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M61" s="2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K62" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="L62" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M62" s="2" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="L63" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M63" s="2" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K64" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="L64" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M64" s="2" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="L65" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M65" s="2" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K66" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="L66" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M66" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M57" xr:uid="{46CAB5D0-DD2F-49FB-AFEA-6E98DB518A23}"/>
+  <autoFilter ref="A1:M66" xr:uid="{7F76AB62-8539-4782-B524-35130B55FA14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M3-T10 (review PASS, Sonnet) - review record, ticket archived, tokens.md section 8 top-inset rule, follow-ups, tracker; STATUS for the 2026-10-07 batch 2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{42696C09-BDFD-40F3-990E-6C4F34A957F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B750B270-1B58-4D73-A5F6-CD2A0532C7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{27DD5107-9878-42E7-9D82-4749B6B52550}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{3888DE25-676E-4C23-B4FD-2CF529742B1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$67</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="474">
   <si>
     <t>ID</t>
   </si>
@@ -1449,6 +1449,21 @@
   </si>
   <si>
     <t>Review PASS WITH FIXES (format) then PASS; follow-up: vitest dist and per-app run</t>
+  </si>
+  <si>
+    <t>M3-T10</t>
+  </si>
+  <si>
+    <t>Layout</t>
+  </si>
+  <si>
+    <t>Top safe-area inset on every screen</t>
+  </si>
+  <si>
+    <t>Done 2026-10-07 (c825350)</t>
+  </si>
+  <si>
+    <t>Review PASS; device pass owed on notched phones</t>
   </si>
 </sst>
 </file>
@@ -1839,8 +1854,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F76AB62-8539-4782-B524-35130B55FA14}">
-  <dimension ref="A1:M66"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E467CF24-153B-47DD-8B48-DF7D9B07E1CB}">
+  <dimension ref="A1:M67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -4544,8 +4559,49 @@
         <v>468</v>
       </c>
     </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A67" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="J67" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="K67" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="L67" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M67" s="2" t="s">
+        <v>473</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M66" xr:uid="{7F76AB62-8539-4782-B524-35130B55FA14}"/>
+  <autoFilter ref="A1:M67" xr:uid="{E467CF24-153B-47DD-8B48-DF7D9B07E1CB}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: Dean's diet list and menu-driven shopping (PO 2026-10-08) - D-024 partial ratification (row 6 and Plan ahead in MVP, row 10 colour still with Dean), D-031 diet preferences sorted list, PRD and domain model updated, ticket M3-E0-T5 (prototype v6: Plan ahead, diet picker, origin band), STATUS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B750B270-1B58-4D73-A5F6-CD2A0532C7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3E23C3B-E17F-443D-8A63-3F15AE3B91EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{3888DE25-676E-4C23-B4FD-2CF529742B1D}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="38700" windowHeight="15345" xr2:uid="{9F87E0AD-A517-4912-927F-647C6484B7BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$68</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="482">
   <si>
     <t>ID</t>
   </si>
@@ -446,10 +446,10 @@
     <t>none</t>
   </si>
   <si>
-    <t>In progress - dispatched 2026-10-07</t>
-  </si>
-  <si>
-    <t>From the impeccable critique of v4 (24/40); PO picked the three P1s; PO sees v5 before acceptance</t>
+    <t>Done - accepted &amp; squash-merged 2026-10-08</t>
+  </si>
+  <si>
+    <t>Review: PASS WITH FIXES -&gt; parallel fix passes merged -&gt; re-check FAIL (focus halo) -&gt; re-check PASS; PO approved v5 2026-10-08; squash 3069d8c; detector 124 -&gt; 29</t>
   </si>
   <si>
     <t>M2</t>
@@ -1464,6 +1464,30 @@
   </si>
   <si>
     <t>Review PASS; device pass owed on notched phones</t>
+  </si>
+  <si>
+    <t>M3-E0-T5</t>
+  </si>
+  <si>
+    <t>M3-E0 UX design</t>
+  </si>
+  <si>
+    <t>Prototype v6: Menu Plan ahead, diet picker, shopping origin band</t>
+  </si>
+  <si>
+    <t>Design</t>
+  </si>
+  <si>
+    <t>Prototype HTML with the impeccable skill</t>
+  </si>
+  <si>
+    <t>Diet and allergy copy side by side; gap shown as deterministic</t>
+  </si>
+  <si>
+    <t>Ready 2026-10-08</t>
+  </si>
+  <si>
+    <t>From Dean 2026-10-07; D-024 partial ratification and D-031</t>
   </si>
 </sst>
 </file>
@@ -1854,8 +1878,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E467CF24-153B-47DD-8B48-DF7D9B07E1CB}">
-  <dimension ref="A1:M67"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDBE8FF9-9716-4147-B781-31263C038A17}">
+  <dimension ref="A1:M68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -4600,8 +4624,49 @@
         <v>473</v>
       </c>
     </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A68" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="J68" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="K68" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="L68" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M68" s="2" t="s">
+        <v>481</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M67" xr:uid="{E467CF24-153B-47DD-8B48-DF7D9B07E1CB}"/>
+  <autoFilter ref="A1:M68" xr:uid="{CDBE8FF9-9716-4147-B781-31263C038A17}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(tracker): regenerate xlsx for M3-E0-T7
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\06_Smart-Kitchen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3E23C3B-E17F-443D-8A63-3F15AE3B91EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A60BBBB-85F3-4AF0-B87A-36C5D5A07CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="38700" windowHeight="15345" xr2:uid="{9F87E0AD-A517-4912-927F-647C6484B7BD}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{35C32CB3-ADD0-4B28-AA45-CCF3F68FCB38}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Backlog!$A$1:$M$69</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="887" uniqueCount="489">
   <si>
     <t>ID</t>
   </si>
@@ -1488,6 +1488,27 @@
   </si>
   <si>
     <t>From Dean 2026-10-07; D-024 partial ratification and D-031</t>
+  </si>
+  <si>
+    <t>M3-E0-T7</t>
+  </si>
+  <si>
+    <t>KitchenSmart design kit: DESIGN.md, light and dark token previews, README (from v6)</t>
+  </si>
+  <si>
+    <t>Transcribe v6 values with the impeccable skill</t>
+  </si>
+  <si>
+    <t>No rule-23 surface; values and safety layer checked against v6 and D-021</t>
+  </si>
+  <si>
+    <t>M3-E0-T6</t>
+  </si>
+  <si>
+    <t>Ready 2026-10-14</t>
+  </si>
+  <si>
+    <t>Andy request; impeccable detect QC on both previews; M3-T13 now depends on it</t>
   </si>
 </sst>
 </file>
@@ -1878,8 +1899,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDBE8FF9-9716-4147-B781-31263C038A17}">
-  <dimension ref="A1:M68"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9277EE5E-B622-4C0D-9169-C59E6D6C929F}">
+  <dimension ref="A1:M69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -4665,8 +4686,49 @@
         <v>481</v>
       </c>
     </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="K69" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="L69" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="M69" s="2" t="s">
+        <v>488</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M68" xr:uid="{CDBE8FF9-9716-4147-B781-31263C038A17}"/>
+  <autoFilter ref="A1:M69" xr:uid="{9277EE5E-B622-4C0D-9169-C59E6D6C929F}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>